<commit_message>
Updated script to use key pair auth and added error handeling to roller_downloader also updated the readme and requirements
</commit_message>
<xml_diff>
--- a/data/output/revenue_comparison.xlsx
+++ b/data/output/revenue_comparison.xlsx
@@ -455,7 +455,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -466,10 +466,10 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>2776.2747</v>
+        <v>6962.8017</v>
       </c>
       <c r="E2" t="n">
-        <v>2776.2747</v>
+        <v>6962.8017</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -479,7 +479,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -487,10 +487,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1552.09</v>
+        <v>4895.49</v>
       </c>
       <c r="D3" t="n">
-        <v>1552.09</v>
+        <v>4895.49</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
@@ -503,7 +503,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -511,13 +511,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>387.82</v>
+        <v>1235.46</v>
       </c>
       <c r="D4" t="n">
-        <v>387.8168</v>
+        <v>1235.4622</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.003199999999992542</v>
+        <v>0.002199999999902502</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -527,7 +527,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -535,13 +535,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>3077.63</v>
+        <v>2863.14</v>
       </c>
       <c r="D5" t="n">
-        <v>3077.626</v>
+        <v>2863.1435</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.003999999999905413</v>
+        <v>0.003500000000258296</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -551,7 +551,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -559,13 +559,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>2891.69</v>
+        <v>2029.27</v>
       </c>
       <c r="D6" t="n">
-        <v>2891.6885</v>
+        <v>2029.2686</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.001499999999850843</v>
+        <v>-0.001400000000103319</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -575,7 +575,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -583,13 +583,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>3215.74</v>
+        <v>3842.72</v>
       </c>
       <c r="D7" t="n">
-        <v>3215.74</v>
+        <v>3842.724</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>0.00400000000036016</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -599,7 +599,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -607,13 +607,13 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>4334.25</v>
+        <v>4812.03</v>
       </c>
       <c r="D8" t="n">
-        <v>4334.25</v>
+        <v>4812.0297</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>-0.0002999999996973202</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -623,7 +623,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -631,10 +631,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>4801</v>
+        <v>43900</v>
       </c>
       <c r="D9" t="n">
-        <v>4801</v>
+        <v>43900</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
@@ -647,7 +647,7 @@
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -655,13 +655,13 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1920.42</v>
+        <v>3713.63</v>
       </c>
       <c r="D10" t="n">
-        <v>1920.4245</v>
+        <v>3713.6334</v>
       </c>
       <c r="E10" t="n">
-        <v>0.004500000000007276</v>
+        <v>0.003399999999601278</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -671,7 +671,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -679,13 +679,13 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>2936.67</v>
+        <v>9306.809999999999</v>
       </c>
       <c r="D11" t="n">
-        <v>2936.6679</v>
+        <v>9306.811</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.002099999999700231</v>
+        <v>0.001000000000203727</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -695,7 +695,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -703,13 +703,13 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>6376.36</v>
+        <v>12122.84</v>
       </c>
       <c r="D12" t="n">
-        <v>6376.3585</v>
+        <v>12122.8389</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.001499999999396096</v>
+        <v>-0.001100000001315493</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -719,7 +719,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -727,13 +727,13 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>3341.2</v>
+        <v>4040.07</v>
       </c>
       <c r="D13" t="n">
-        <v>3341.1983</v>
+        <v>4040.0734</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.001699999999800639</v>
+        <v>0.003400000000056025</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -743,7 +743,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -751,13 +751,13 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>2534.3</v>
+        <v>18126.65</v>
       </c>
       <c r="D14" t="n">
-        <v>2534.3039</v>
+        <v>18126.6545</v>
       </c>
       <c r="E14" t="n">
-        <v>0.003900000000157888</v>
+        <v>0.004499999999097781</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -767,7 +767,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -775,13 +775,13 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2720.22</v>
+        <v>5510.69</v>
       </c>
       <c r="D15" t="n">
-        <v>2720.2215</v>
+        <v>5510.6858</v>
       </c>
       <c r="E15" t="n">
-        <v>0.00150000000030559</v>
+        <v>-0.004199999999400461</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -791,7 +791,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -799,13 +799,13 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>4232.88</v>
+        <v>2609.72</v>
       </c>
       <c r="D16" t="n">
-        <v>4232.8819</v>
+        <v>2609.7198</v>
       </c>
       <c r="E16" t="n">
-        <v>0.001900000000205182</v>
+        <v>-0.0001999999999497959</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -815,7 +815,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -823,13 +823,13 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1345.78</v>
+        <v>5203.05</v>
       </c>
       <c r="D17" t="n">
-        <v>1345.7839</v>
+        <v>5203.0522</v>
       </c>
       <c r="E17" t="n">
-        <v>0.003899999999930515</v>
+        <v>0.002199999999902502</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -839,7 +839,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -847,13 +847,13 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>2015.59</v>
+        <v>4411.59</v>
       </c>
       <c r="D18" t="n">
-        <v>2015.5852</v>
+        <v>4411.5921</v>
       </c>
       <c r="E18" t="n">
-        <v>-0.00479999999993197</v>
+        <v>0.002099999999700231</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -863,7 +863,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -871,13 +871,13 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>7794.57</v>
+        <v>13837.58</v>
       </c>
       <c r="D19" t="n">
-        <v>7794.57</v>
+        <v>13837.5794</v>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>-0.0005999999993946403</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -887,7 +887,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -895,13 +895,13 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2222.7</v>
+        <v>4460.64</v>
       </c>
       <c r="D20" t="n">
-        <v>2222.7013</v>
+        <v>4460.637400000001</v>
       </c>
       <c r="E20" t="n">
-        <v>0.001299999999901047</v>
+        <v>-0.002599999999802094</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -911,7 +911,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -919,13 +919,13 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>2214.63</v>
+        <v>6814.76</v>
       </c>
       <c r="D21" t="n">
-        <v>2214.6285</v>
+        <v>6814.762600000001</v>
       </c>
       <c r="E21" t="n">
-        <v>-0.00150000000030559</v>
+        <v>0.002600000000711589</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -935,7 +935,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -943,13 +943,13 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>4015.84</v>
+        <v>3632.22</v>
       </c>
       <c r="D22" t="n">
-        <v>4015.8357</v>
+        <v>3632.2241</v>
       </c>
       <c r="E22" t="n">
-        <v>-0.00430000000005748</v>
+        <v>0.004100000000107684</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -959,7 +959,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -967,13 +967,13 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1848.35</v>
+        <v>2583.83</v>
       </c>
       <c r="D23" t="n">
-        <v>1848.3466</v>
+        <v>2583.8338</v>
       </c>
       <c r="E23" t="n">
-        <v>-0.003399999999828651</v>
+        <v>0.003799999999955617</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -983,7 +983,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -991,13 +991,13 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>2403.8</v>
+        <v>6469.53</v>
       </c>
       <c r="D24" t="n">
-        <v>2403.8021</v>
+        <v>6469.531599999999</v>
       </c>
       <c r="E24" t="n">
-        <v>0.002099999999700231</v>
+        <v>0.001599999999598367</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -1007,7 +1007,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -1015,23 +1015,23 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>2637.08</v>
+        <v>4251.29</v>
       </c>
       <c r="D25" t="n">
-        <v>2637.08</v>
+        <v>4226.3</v>
       </c>
       <c r="E25" t="n">
-        <v>0</v>
+        <v>-24.98999999999978</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Match</t>
+          <t>Mismatch</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -1039,13 +1039,13 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>3132.11</v>
+        <v>4623.47</v>
       </c>
       <c r="D26" t="n">
-        <v>3132.1061</v>
+        <v>4623.4701</v>
       </c>
       <c r="E26" t="n">
-        <v>-0.003900000000157888</v>
+        <v>9.999999929277692e-05</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -1055,7 +1055,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -1063,13 +1063,13 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>2356.55</v>
+        <v>13883.06</v>
       </c>
       <c r="D27" t="n">
-        <v>2356.553</v>
+        <v>13883.0551</v>
       </c>
       <c r="E27" t="n">
-        <v>0.002999999999701686</v>
+        <v>-0.004899999998087878</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -1079,7 +1079,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -1087,13 +1087,13 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>2192.92</v>
+        <v>6836.81</v>
       </c>
       <c r="D28" t="n">
-        <v>2192.9162</v>
+        <v>6836.810100000001</v>
       </c>
       <c r="E28" t="n">
-        <v>-0.003799999999955617</v>
+        <v>0.0001000000002022716</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -1103,7 +1103,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -1111,13 +1111,13 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>3229.41</v>
+        <v>6350.76</v>
       </c>
       <c r="D29" t="n">
-        <v>3229.4088</v>
+        <v>6350.7634</v>
       </c>
       <c r="E29" t="n">
-        <v>-0.001199999999698775</v>
+        <v>0.003399999999601278</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -1127,7 +1127,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -1135,13 +1135,13 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>4173.9</v>
+        <v>11408.23</v>
       </c>
       <c r="D30" t="n">
-        <v>4173.8999</v>
+        <v>11408.233</v>
       </c>
       <c r="E30" t="n">
-        <v>-9.999999929277692e-05</v>
+        <v>0.00300000000061118</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -1151,7 +1151,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -1159,13 +1159,13 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>7668.9</v>
+        <v>13632.59</v>
       </c>
       <c r="D31" t="n">
-        <v>7668.9011</v>
+        <v>13632.5929</v>
       </c>
       <c r="E31" t="n">
-        <v>0.001100000000405998</v>
+        <v>0.002899999999499414</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -1175,7 +1175,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -1183,13 +1183,13 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>2805.87</v>
+        <v>4067.21</v>
       </c>
       <c r="D32" t="n">
-        <v>2805.8668</v>
+        <v>4067.2114</v>
       </c>
       <c r="E32" t="n">
-        <v>-0.003199999999651482</v>
+        <v>0.001400000000103319</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -1199,7 +1199,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -1207,13 +1207,13 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>2887.92</v>
+        <v>8936.32</v>
       </c>
       <c r="D33" t="n">
-        <v>2887.9194</v>
+        <v>8936.322699999999</v>
       </c>
       <c r="E33" t="n">
-        <v>-0.000600000000304135</v>
+        <v>0.002699999999094871</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -1223,7 +1223,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -1231,13 +1231,13 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1786.08</v>
+        <v>4408.47</v>
       </c>
       <c r="D34" t="n">
-        <v>1786.08</v>
+        <v>4408.4699</v>
       </c>
       <c r="E34" t="n">
-        <v>0</v>
+        <v>-0.0001000000002022716</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -1247,7 +1247,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -1255,13 +1255,13 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>2144.41</v>
+        <v>2990.97</v>
       </c>
       <c r="D35" t="n">
-        <v>2144.41</v>
+        <v>2990.97</v>
       </c>
       <c r="E35" t="n">
-        <v>0</v>
+        <v>4.547473508864641e-13</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -1271,7 +1271,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -1279,13 +1279,13 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>1863</v>
+        <v>2895.38</v>
       </c>
       <c r="D36" t="n">
-        <v>1862.9956</v>
+        <v>2895.3848</v>
       </c>
       <c r="E36" t="n">
-        <v>-0.004400000000032378</v>
+        <v>0.004800000000159343</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -1295,7 +1295,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -1303,13 +1303,13 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>5507.16</v>
+        <v>30646.34</v>
       </c>
       <c r="D37" t="n">
-        <v>5507.1605</v>
+        <v>30646.3391</v>
       </c>
       <c r="E37" t="n">
-        <v>0.0005000000001018634</v>
+        <v>-0.0009000000027299393</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
@@ -1319,7 +1319,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -1327,13 +1327,13 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>2782.31</v>
+        <v>8112.29</v>
       </c>
       <c r="D38" t="n">
-        <v>2782.3125</v>
+        <v>8112.2859</v>
       </c>
       <c r="E38" t="n">
-        <v>0.00250000000005457</v>
+        <v>-0.004100000000107684</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
@@ -1343,7 +1343,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -1351,13 +1351,13 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>5288.63</v>
+        <v>6864.92</v>
       </c>
       <c r="D39" t="n">
-        <v>5288.6318</v>
+        <v>6864.9221</v>
       </c>
       <c r="E39" t="n">
-        <v>0.00180000000000291</v>
+        <v>0.002099999999700231</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
@@ -1367,7 +1367,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -1375,13 +1375,13 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>5008.69</v>
+        <v>20669.13</v>
       </c>
       <c r="D40" t="n">
-        <v>5008.6899</v>
+        <v>20669.1294</v>
       </c>
       <c r="E40" t="n">
-        <v>-9.999999929277692e-05</v>
+        <v>-0.0005999999993946403</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
@@ -1391,7 +1391,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -1399,13 +1399,13 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>3505.56</v>
+        <v>17580.33</v>
       </c>
       <c r="D41" t="n">
-        <v>3505.558500000001</v>
+        <v>17580.3301</v>
       </c>
       <c r="E41" t="n">
-        <v>-0.001499999999396096</v>
+        <v>9.999999747378752e-05</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
@@ -1415,7 +1415,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -1423,13 +1423,13 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>5139.68</v>
+        <v>7644.91</v>
       </c>
       <c r="D42" t="n">
-        <v>5139.682</v>
+        <v>7644.9067</v>
       </c>
       <c r="E42" t="n">
-        <v>0.001999999999497959</v>
+        <v>-0.003300000000308501</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
@@ -1439,7 +1439,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -1447,13 +1447,13 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>2494.89</v>
+        <v>5514.33</v>
       </c>
       <c r="D43" t="n">
-        <v>2494.8894</v>
+        <v>5514.3255</v>
       </c>
       <c r="E43" t="n">
-        <v>-0.0005999999998493877</v>
+        <v>-0.004500000000007276</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
@@ -1463,7 +1463,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -1471,13 +1471,13 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>3155.27</v>
+        <v>9423.469999999999</v>
       </c>
       <c r="D44" t="n">
-        <v>3155.2676</v>
+        <v>9423.4701</v>
       </c>
       <c r="E44" t="n">
-        <v>-0.002399999999852298</v>
+        <v>0.0001000000011117663</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
@@ -1487,7 +1487,7 @@
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -1495,13 +1495,13 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>2181.44</v>
+        <v>4677.27</v>
       </c>
       <c r="D45" t="n">
-        <v>2181.4379</v>
+        <v>4677.2734</v>
       </c>
       <c r="E45" t="n">
-        <v>-0.002100000000154978</v>
+        <v>0.003399999999601278</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
@@ -1511,7 +1511,7 @@
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
@@ -1519,13 +1519,13 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>479.01</v>
+        <v>3431.89</v>
       </c>
       <c r="D46" t="n">
-        <v>479.0149</v>
+        <v>3431.8897</v>
       </c>
       <c r="E46" t="n">
-        <v>0.004899999999963711</v>
+        <v>-0.0003000000001520675</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
@@ -1535,7 +1535,7 @@
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -1543,13 +1543,13 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>3722.98</v>
+        <v>13101.72</v>
       </c>
       <c r="D47" t="n">
-        <v>3722.98</v>
+        <v>13101.7178</v>
       </c>
       <c r="E47" t="n">
-        <v>-4.547473508864641e-13</v>
+        <v>-0.002199999998993007</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
@@ -1559,7 +1559,7 @@
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
@@ -1567,13 +1567,13 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>3931.08</v>
+        <v>4346.74</v>
       </c>
       <c r="D48" t="n">
-        <v>3931.0829</v>
+        <v>4346.737599999999</v>
       </c>
       <c r="E48" t="n">
-        <v>0.002899999999954161</v>
+        <v>-0.002400000000307045</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
@@ -1583,7 +1583,7 @@
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
@@ -1591,13 +1591,13 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>5002.61</v>
+        <v>12953.84</v>
       </c>
       <c r="D49" t="n">
-        <v>5002.6105</v>
+        <v>12953.8394</v>
       </c>
       <c r="E49" t="n">
-        <v>0.0005000000001018634</v>
+        <v>-0.0006000000012136297</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
@@ -1607,7 +1607,7 @@
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
@@ -1615,13 +1615,13 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>2928.09</v>
+        <v>9277.459999999999</v>
       </c>
       <c r="D50" t="n">
-        <v>2928.0863</v>
+        <v>9277.455599999999</v>
       </c>
       <c r="E50" t="n">
-        <v>-0.003700000000208092</v>
+        <v>-0.004399999999805004</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
@@ -1631,7 +1631,7 @@
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
@@ -1639,13 +1639,13 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>3984.82</v>
+        <v>5197.22</v>
       </c>
       <c r="D51" t="n">
-        <v>3984.823</v>
+        <v>5197.2196</v>
       </c>
       <c r="E51" t="n">
-        <v>0.002999999999701686</v>
+        <v>-0.0003999999998995918</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
@@ -1655,7 +1655,7 @@
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
@@ -1663,13 +1663,13 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>2889.18</v>
+        <v>7848.93</v>
       </c>
       <c r="D52" t="n">
-        <v>2889.1836</v>
+        <v>7848.928199999998</v>
       </c>
       <c r="E52" t="n">
-        <v>0.003600000000005821</v>
+        <v>-0.0018000000018219</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
@@ -1679,7 +1679,7 @@
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
@@ -1687,13 +1687,13 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>1434.78</v>
+        <v>2495.01</v>
       </c>
       <c r="D53" t="n">
-        <v>1434.781</v>
+        <v>2495.0053</v>
       </c>
       <c r="E53" t="n">
-        <v>0.0009999999999763531</v>
+        <v>-0.004700000000411819</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
@@ -1703,7 +1703,7 @@
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
@@ -1711,13 +1711,13 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>2944.98</v>
+        <v>6686.93</v>
       </c>
       <c r="D54" t="n">
-        <v>2944.9818</v>
+        <v>6686.933999999999</v>
       </c>
       <c r="E54" t="n">
-        <v>0.00180000000000291</v>
+        <v>0.003999999998995918</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
@@ -1727,7 +1727,7 @@
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
@@ -1735,13 +1735,13 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>4779.7</v>
+        <v>8344.24</v>
       </c>
       <c r="D55" t="n">
-        <v>4779.7038</v>
+        <v>8344.239399999999</v>
       </c>
       <c r="E55" t="n">
-        <v>0.003800000000410364</v>
+        <v>-0.0006000000012136297</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
@@ -1751,7 +1751,7 @@
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
@@ -1759,13 +1759,13 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>6885.74</v>
+        <v>11474.17</v>
       </c>
       <c r="D56" t="n">
-        <v>6885.7425</v>
+        <v>11474.17</v>
       </c>
       <c r="E56" t="n">
-        <v>0.002500000000509317</v>
+        <v>-1.818989403545856e-12</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
@@ -1775,7 +1775,7 @@
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
@@ -1783,13 +1783,13 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>785.24</v>
+        <v>970.77</v>
       </c>
       <c r="D57" t="n">
-        <v>785.2379999999999</v>
+        <v>970.7706999999999</v>
       </c>
       <c r="E57" t="n">
-        <v>-0.002000000000066393</v>
+        <v>0.0006999999999379725</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
@@ -1799,7 +1799,7 @@
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
@@ -1807,23 +1807,23 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>6508.08</v>
+        <v>26273.91</v>
       </c>
       <c r="D58" t="n">
-        <v>6508.0815</v>
+        <v>26364.527</v>
       </c>
       <c r="E58" t="n">
-        <v>0.00150000000030559</v>
+        <v>90.61700000000201</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Match</t>
+          <t>Mismatch</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
@@ -1831,13 +1831,13 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>5462.33</v>
+        <v>9975.18</v>
       </c>
       <c r="D59" t="n">
-        <v>5462.328</v>
+        <v>9975.180900000001</v>
       </c>
       <c r="E59" t="n">
-        <v>-0.001999999999497959</v>
+        <v>0.0009000000009109499</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
@@ -1847,7 +1847,7 @@
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
@@ -1855,13 +1855,13 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>2790.15</v>
+        <v>6147.58</v>
       </c>
       <c r="D60" t="n">
-        <v>2790.1517</v>
+        <v>6147.5838</v>
       </c>
       <c r="E60" t="n">
-        <v>0.001699999999800639</v>
+        <v>0.003800000000410364</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
@@ -1871,7 +1871,7 @@
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
@@ -1879,13 +1879,13 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>1895.66</v>
+        <v>3021.75</v>
       </c>
       <c r="D61" t="n">
-        <v>1895.6621</v>
+        <v>3021.7542</v>
       </c>
       <c r="E61" t="n">
-        <v>0.002099999999927604</v>
+        <v>0.004199999999855208</v>
       </c>
       <c r="F61" t="inlineStr">
         <is>
@@ -1895,7 +1895,7 @@
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
@@ -1903,13 +1903,13 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>1431.18</v>
+        <v>6322.5</v>
       </c>
       <c r="D62" t="n">
-        <v>1431.1805</v>
+        <v>6322.501</v>
       </c>
       <c r="E62" t="n">
-        <v>0.0004999999998744897</v>
+        <v>0.001000000000203727</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
@@ -1919,7 +1919,7 @@
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
@@ -1927,13 +1927,13 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>4976.93</v>
+        <v>14909.06</v>
       </c>
       <c r="D63" t="n">
-        <v>4976.9283</v>
+        <v>14909.056</v>
       </c>
       <c r="E63" t="n">
-        <v>-0.001700000000710133</v>
+        <v>-0.003999999998995918</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
@@ -1943,7 +1943,7 @@
     </row>
     <row r="64">
       <c r="A64" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
@@ -1951,13 +1951,13 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>2492.03</v>
+        <v>7145.87</v>
       </c>
       <c r="D64" t="n">
-        <v>2492.03</v>
+        <v>7145.874199999999</v>
       </c>
       <c r="E64" t="n">
-        <v>-4.547473508864641e-13</v>
+        <v>0.004199999999400461</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
@@ -1967,7 +1967,7 @@
     </row>
     <row r="65">
       <c r="A65" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
@@ -1975,13 +1975,13 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>3103.48</v>
+        <v>6021.58</v>
       </c>
       <c r="D65" t="n">
-        <v>3103.4755</v>
+        <v>6021.578299999999</v>
       </c>
       <c r="E65" t="n">
-        <v>-0.004500000000007276</v>
+        <v>-0.001700000000710133</v>
       </c>
       <c r="F65" t="inlineStr">
         <is>
@@ -1991,7 +1991,7 @@
     </row>
     <row r="66">
       <c r="A66" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
@@ -1999,13 +1999,13 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>1533.97</v>
+        <v>2765.61</v>
       </c>
       <c r="D66" t="n">
-        <v>1533.9684</v>
+        <v>2765.6107</v>
       </c>
       <c r="E66" t="n">
-        <v>-0.001599999999825741</v>
+        <v>0.0007000000000516593</v>
       </c>
       <c r="F66" t="inlineStr">
         <is>
@@ -2015,7 +2015,7 @@
     </row>
     <row r="67">
       <c r="A67" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
@@ -2023,13 +2023,13 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>1201.01</v>
+        <v>4946.34</v>
       </c>
       <c r="D67" t="n">
-        <v>1201.0126</v>
+        <v>4946.3394</v>
       </c>
       <c r="E67" t="n">
-        <v>0.002600000000029468</v>
+        <v>-0.000600000000304135</v>
       </c>
       <c r="F67" t="inlineStr">
         <is>
@@ -2039,7 +2039,7 @@
     </row>
     <row r="68">
       <c r="A68" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
@@ -2047,13 +2047,13 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>1889.16</v>
+        <v>4502.54</v>
       </c>
       <c r="D68" t="n">
-        <v>1889.1594</v>
+        <v>4502.5421</v>
       </c>
       <c r="E68" t="n">
-        <v>-0.0006000000000767614</v>
+        <v>0.002099999999700231</v>
       </c>
       <c r="F68" t="inlineStr">
         <is>
@@ -2063,7 +2063,7 @@
     </row>
     <row r="69">
       <c r="A69" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
@@ -2071,13 +2071,13 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>3717.26</v>
+        <v>14109.33</v>
       </c>
       <c r="D69" t="n">
-        <v>3717.2585</v>
+        <v>14109.331</v>
       </c>
       <c r="E69" t="n">
-        <v>-0.00150000000030559</v>
+        <v>0.001000000000203727</v>
       </c>
       <c r="F69" t="inlineStr">
         <is>
@@ -2087,7 +2087,7 @@
     </row>
     <row r="70">
       <c r="A70" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
@@ -2095,13 +2095,13 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>9083.469999999999</v>
+        <v>22093.13</v>
       </c>
       <c r="D70" t="n">
-        <v>9083.470600000001</v>
+        <v>22093.1324</v>
       </c>
       <c r="E70" t="n">
-        <v>0.0006000000012136297</v>
+        <v>0.002399999997578561</v>
       </c>
       <c r="F70" t="inlineStr">
         <is>
@@ -2111,7 +2111,7 @@
     </row>
     <row r="71">
       <c r="A71" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
@@ -2119,13 +2119,13 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>4201.9</v>
+        <v>8694.700000000001</v>
       </c>
       <c r="D71" t="n">
-        <v>4201.9046</v>
+        <v>8694.697900000001</v>
       </c>
       <c r="E71" t="n">
-        <v>0.004600000000209548</v>
+        <v>-0.002099999999700231</v>
       </c>
       <c r="F71" t="inlineStr">
         <is>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="72">
       <c r="A72" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
@@ -2143,13 +2143,13 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>3117.85</v>
+        <v>9824.110000000001</v>
       </c>
       <c r="D72" t="n">
-        <v>3117.8451</v>
+        <v>9824.107199999999</v>
       </c>
       <c r="E72" t="n">
-        <v>-0.004899999999906868</v>
+        <v>-0.002800000002025627</v>
       </c>
       <c r="F72" t="inlineStr">
         <is>
@@ -2159,7 +2159,7 @@
     </row>
     <row r="73">
       <c r="A73" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
@@ -2167,23 +2167,23 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>2240.93</v>
+        <v>3888.3</v>
       </c>
       <c r="D73" t="n">
-        <v>2240.93</v>
+        <v>3840.32</v>
       </c>
       <c r="E73" t="n">
-        <v>0</v>
+        <v>-47.98000000000047</v>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Match</t>
+          <t>Mismatch</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
@@ -2191,13 +2191,13 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>3189.11</v>
+        <v>6887.67</v>
       </c>
       <c r="D74" t="n">
-        <v>3189.1095</v>
+        <v>6887.6705</v>
       </c>
       <c r="E74" t="n">
-        <v>-0.0005000000001018634</v>
+        <v>0.0005000000001018634</v>
       </c>
       <c r="F74" t="inlineStr">
         <is>
@@ -2207,7 +2207,7 @@
     </row>
     <row r="75">
       <c r="A75" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
@@ -2215,13 +2215,13 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>10765.55</v>
+        <v>8967.540000000001</v>
       </c>
       <c r="D75" t="n">
-        <v>11018.9804</v>
+        <v>8983.7212</v>
       </c>
       <c r="E75" t="n">
-        <v>253.4304000000011</v>
+        <v>16.18119999999908</v>
       </c>
       <c r="F75" t="inlineStr">
         <is>
@@ -2231,7 +2231,7 @@
     </row>
     <row r="76">
       <c r="A76" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
@@ -2239,13 +2239,13 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>2185.3</v>
+        <v>3968.6</v>
       </c>
       <c r="D76" t="n">
-        <v>2185.3049</v>
+        <v>3968.5963</v>
       </c>
       <c r="E76" t="n">
-        <v>0.004899999999906868</v>
+        <v>-0.003700000000208092</v>
       </c>
       <c r="F76" t="inlineStr">
         <is>
@@ -2255,7 +2255,7 @@
     </row>
     <row r="77">
       <c r="A77" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
@@ -2263,13 +2263,13 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>1446.37</v>
+        <v>2605.31</v>
       </c>
       <c r="D77" t="n">
-        <v>1446.37</v>
+        <v>2605.3118</v>
       </c>
       <c r="E77" t="n">
-        <v>0</v>
+        <v>0.00180000000000291</v>
       </c>
       <c r="F77" t="inlineStr">
         <is>
@@ -2279,7 +2279,7 @@
     </row>
     <row r="78">
       <c r="A78" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
@@ -2287,13 +2287,13 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>2814.79</v>
+        <v>7298.14</v>
       </c>
       <c r="D78" t="n">
-        <v>2814.7914</v>
+        <v>7298.1446</v>
       </c>
       <c r="E78" t="n">
-        <v>0.001400000000103319</v>
+        <v>0.004599999999300053</v>
       </c>
       <c r="F78" t="inlineStr">
         <is>
@@ -2303,7 +2303,7 @@
     </row>
     <row r="79">
       <c r="A79" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
@@ -2311,13 +2311,13 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>7337.94</v>
+        <v>17555.06</v>
       </c>
       <c r="D79" t="n">
-        <v>7337.9415</v>
+        <v>17555.0565</v>
       </c>
       <c r="E79" t="n">
-        <v>0.00150000000030559</v>
+        <v>-0.003500000002532033</v>
       </c>
       <c r="F79" t="inlineStr">
         <is>
@@ -2327,7 +2327,7 @@
     </row>
     <row r="80">
       <c r="A80" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
@@ -2335,13 +2335,13 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>2873.81</v>
+        <v>9142.059999999999</v>
       </c>
       <c r="D80" t="n">
-        <v>2873.8067</v>
+        <v>9142.060499999998</v>
       </c>
       <c r="E80" t="n">
-        <v>-0.003299999999853753</v>
+        <v>0.000499999998282874</v>
       </c>
       <c r="F80" t="inlineStr">
         <is>
@@ -2351,7 +2351,7 @@
     </row>
     <row r="81">
       <c r="A81" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
@@ -2359,13 +2359,13 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>2024.38</v>
+        <v>18063.83</v>
       </c>
       <c r="D81" t="n">
-        <v>2024.3846</v>
+        <v>18063.8281</v>
       </c>
       <c r="E81" t="n">
-        <v>0.004599999999982174</v>
+        <v>-0.001900000002933666</v>
       </c>
       <c r="F81" t="inlineStr">
         <is>
@@ -2375,7 +2375,7 @@
     </row>
     <row r="82">
       <c r="A82" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
@@ -2383,13 +2383,13 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>4589.54</v>
+        <v>7127.71</v>
       </c>
       <c r="D82" t="n">
-        <v>4589.5437</v>
+        <v>7127.7131</v>
       </c>
       <c r="E82" t="n">
-        <v>0.003700000000208092</v>
+        <v>0.003099999999903957</v>
       </c>
       <c r="F82" t="inlineStr">
         <is>
@@ -2399,7 +2399,7 @@
     </row>
     <row r="83">
       <c r="A83" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
@@ -2407,13 +2407,13 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>3651.98</v>
+        <v>7103.19</v>
       </c>
       <c r="D83" t="n">
-        <v>3651.9842</v>
+        <v>7103.194599999999</v>
       </c>
       <c r="E83" t="n">
-        <v>0.004199999999855208</v>
+        <v>0.004599999999300053</v>
       </c>
       <c r="F83" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     </row>
     <row r="84">
       <c r="A84" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
@@ -2431,13 +2431,13 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>2216.91</v>
+        <v>5081.59</v>
       </c>
       <c r="D84" t="n">
-        <v>2216.9149</v>
+        <v>5081.5877</v>
       </c>
       <c r="E84" t="n">
-        <v>0.004899999999906868</v>
+        <v>-0.002300000000104774</v>
       </c>
       <c r="F84" t="inlineStr">
         <is>
@@ -2447,7 +2447,7 @@
     </row>
     <row r="85">
       <c r="A85" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
@@ -2455,13 +2455,13 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>2174.98</v>
+        <v>2496.33</v>
       </c>
       <c r="D85" t="n">
-        <v>2174.9806</v>
+        <v>2496.3317</v>
       </c>
       <c r="E85" t="n">
-        <v>0.0005999999998493877</v>
+        <v>0.001699999999800639</v>
       </c>
       <c r="F85" t="inlineStr">
         <is>
@@ -2471,7 +2471,7 @@
     </row>
     <row r="86">
       <c r="A86" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
@@ -2479,13 +2479,13 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>4277.75</v>
+        <v>10024.15</v>
       </c>
       <c r="D86" t="n">
-        <v>4277.7454</v>
+        <v>10024.1469</v>
       </c>
       <c r="E86" t="n">
-        <v>-0.004600000000209548</v>
+        <v>-0.003099999998084968</v>
       </c>
       <c r="F86" t="inlineStr">
         <is>
@@ -2495,7 +2495,7 @@
     </row>
     <row r="87">
       <c r="A87" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
@@ -2503,13 +2503,13 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>8938.24</v>
+        <v>13086.02</v>
       </c>
       <c r="D87" t="n">
-        <v>8938.2387</v>
+        <v>13086.0181</v>
       </c>
       <c r="E87" t="n">
-        <v>-0.001299999999901047</v>
+        <v>-0.001900000001114677</v>
       </c>
       <c r="F87" t="inlineStr">
         <is>
@@ -2519,7 +2519,7 @@
     </row>
     <row r="88">
       <c r="A88" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
@@ -2527,13 +2527,13 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>5022.22</v>
+        <v>10428.66</v>
       </c>
       <c r="D88" t="n">
-        <v>5022.2191</v>
+        <v>10428.6631</v>
       </c>
       <c r="E88" t="n">
-        <v>-0.0009000000000014552</v>
+        <v>0.003099999998084968</v>
       </c>
       <c r="F88" t="inlineStr">
         <is>
@@ -2543,7 +2543,7 @@
     </row>
     <row r="89">
       <c r="A89" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
@@ -2551,13 +2551,13 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>3373.11</v>
+        <v>6938.56</v>
       </c>
       <c r="D89" t="n">
-        <v>3373.1061</v>
+        <v>6938.557000000001</v>
       </c>
       <c r="E89" t="n">
-        <v>-0.003900000000157888</v>
+        <v>-0.002999999999701686</v>
       </c>
       <c r="F89" t="inlineStr">
         <is>
@@ -2567,7 +2567,7 @@
     </row>
     <row r="90">
       <c r="A90" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
@@ -2575,13 +2575,13 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>3599.43</v>
+        <v>6221.92</v>
       </c>
       <c r="D90" t="n">
-        <v>3599.4277</v>
+        <v>6221.9221</v>
       </c>
       <c r="E90" t="n">
-        <v>-0.002299999999650026</v>
+        <v>0.002099999999700231</v>
       </c>
       <c r="F90" t="inlineStr">
         <is>
@@ -2591,7 +2591,7 @@
     </row>
     <row r="91">
       <c r="A91" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B91" t="inlineStr">
         <is>
@@ -2599,13 +2599,13 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>6276.02</v>
+        <v>5526.81</v>
       </c>
       <c r="D91" t="n">
-        <v>6276.0189</v>
+        <v>5526.805799999999</v>
       </c>
       <c r="E91" t="n">
-        <v>-0.001100000000405998</v>
+        <v>-0.00420000000121945</v>
       </c>
       <c r="F91" t="inlineStr">
         <is>
@@ -2615,7 +2615,7 @@
     </row>
     <row r="92">
       <c r="A92" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
@@ -2623,13 +2623,13 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>2786.06</v>
+        <v>5940.29</v>
       </c>
       <c r="D92" t="n">
-        <v>2786.0648</v>
+        <v>5940.2898</v>
       </c>
       <c r="E92" t="n">
-        <v>0.004800000000159343</v>
+        <v>-0.0001999999994950485</v>
       </c>
       <c r="F92" t="inlineStr">
         <is>
@@ -2639,7 +2639,7 @@
     </row>
     <row r="93">
       <c r="A93" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
@@ -2647,13 +2647,13 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>2770.03</v>
+        <v>3998.32</v>
       </c>
       <c r="D93" t="n">
-        <v>2770.0254</v>
+        <v>3998.3208</v>
       </c>
       <c r="E93" t="n">
-        <v>-0.0045999999997548</v>
+        <v>0.0007999999997991836</v>
       </c>
       <c r="F93" t="inlineStr">
         <is>
@@ -2663,7 +2663,7 @@
     </row>
     <row r="94">
       <c r="A94" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
@@ -2671,13 +2671,13 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>1106.7</v>
+        <v>4822.33</v>
       </c>
       <c r="D94" t="n">
-        <v>1106.7034</v>
+        <v>4822.3259</v>
       </c>
       <c r="E94" t="n">
-        <v>0.003400000000056025</v>
+        <v>-0.004100000000107684</v>
       </c>
       <c r="F94" t="inlineStr">
         <is>
@@ -2687,7 +2687,7 @@
     </row>
     <row r="95">
       <c r="A95" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
@@ -2695,13 +2695,13 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>2572.43</v>
+        <v>2073.83</v>
       </c>
       <c r="D95" t="n">
-        <v>2572.4256</v>
+        <v>2073.8291</v>
       </c>
       <c r="E95" t="n">
-        <v>-0.004399999999805004</v>
+        <v>-0.0009000000000014552</v>
       </c>
       <c r="F95" t="inlineStr">
         <is>
@@ -2711,7 +2711,7 @@
     </row>
     <row r="96">
       <c r="A96" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
@@ -2719,13 +2719,13 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>5069.4</v>
+        <v>6893.56</v>
       </c>
       <c r="D96" t="n">
-        <v>5069.4028</v>
+        <v>6893.561899999999</v>
       </c>
       <c r="E96" t="n">
-        <v>0.002800000000206637</v>
+        <v>0.001899999998386193</v>
       </c>
       <c r="F96" t="inlineStr">
         <is>
@@ -2735,7 +2735,7 @@
     </row>
     <row r="97">
       <c r="A97" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
@@ -2743,13 +2743,13 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>1249.77</v>
+        <v>2036.77</v>
       </c>
       <c r="D97" t="n">
-        <v>1249.7704</v>
+        <v>2036.7718</v>
       </c>
       <c r="E97" t="n">
-        <v>0.0003999999998995918</v>
+        <v>0.00180000000000291</v>
       </c>
       <c r="F97" t="inlineStr">
         <is>
@@ -2759,7 +2759,7 @@
     </row>
     <row r="98">
       <c r="A98" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
@@ -2767,23 +2767,23 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>6244.95</v>
+        <v>13449.81</v>
       </c>
       <c r="D98" t="n">
-        <v>6244.947400000001</v>
+        <v>13544.7547</v>
       </c>
       <c r="E98" t="n">
-        <v>-0.002599999998892599</v>
+        <v>94.94470000000001</v>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>Match</t>
+          <t>Mismatch</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
@@ -2791,13 +2791,13 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>2252.33</v>
+        <v>8050.28</v>
       </c>
       <c r="D99" t="n">
-        <v>2252.3344</v>
+        <v>8050.2823</v>
       </c>
       <c r="E99" t="n">
-        <v>0.004399999999805004</v>
+        <v>0.002300000000104774</v>
       </c>
       <c r="F99" t="inlineStr">
         <is>
@@ -2807,7 +2807,7 @@
     </row>
     <row r="100">
       <c r="A100" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
@@ -2815,13 +2815,13 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>627.73</v>
+        <v>3048.9</v>
       </c>
       <c r="D100" t="n">
-        <v>627.7253000000001</v>
+        <v>3048.9047</v>
       </c>
       <c r="E100" t="n">
-        <v>-0.004699999999957072</v>
+        <v>0.004699999999502324</v>
       </c>
       <c r="F100" t="inlineStr">
         <is>
@@ -2831,7 +2831,7 @@
     </row>
     <row r="101">
       <c r="A101" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
@@ -2839,13 +2839,13 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>2653.28</v>
+        <v>7216.29</v>
       </c>
       <c r="D101" t="n">
-        <v>2653.2821</v>
+        <v>7216.2873</v>
       </c>
       <c r="E101" t="n">
-        <v>0.002099999999700231</v>
+        <v>-0.002700000000004366</v>
       </c>
       <c r="F101" t="inlineStr">
         <is>
@@ -2855,7 +2855,7 @@
     </row>
     <row r="102">
       <c r="A102" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
@@ -2863,13 +2863,13 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>3937.59</v>
+        <v>12992.68</v>
       </c>
       <c r="D102" t="n">
-        <v>3937.5941</v>
+        <v>12992.678</v>
       </c>
       <c r="E102" t="n">
-        <v>0.004099999999652937</v>
+        <v>-0.002000000002226443</v>
       </c>
       <c r="F102" t="inlineStr">
         <is>
@@ -2879,7 +2879,7 @@
     </row>
     <row r="103">
       <c r="A103" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
@@ -2887,13 +2887,13 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>2687.16</v>
+        <v>10464.08</v>
       </c>
       <c r="D103" t="n">
-        <v>2687.1615</v>
+        <v>10464.0804</v>
       </c>
       <c r="E103" t="n">
-        <v>0.001499999999850843</v>
+        <v>0.0004000000008090865</v>
       </c>
       <c r="F103" t="inlineStr">
         <is>
@@ -2903,7 +2903,7 @@
     </row>
     <row r="104">
       <c r="A104" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
@@ -2911,13 +2911,13 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>3366.76</v>
+        <v>11346.58</v>
       </c>
       <c r="D104" t="n">
-        <v>3366.76</v>
+        <v>11346.5825</v>
       </c>
       <c r="E104" t="n">
-        <v>0</v>
+        <v>0.002500000000509317</v>
       </c>
       <c r="F104" t="inlineStr">
         <is>
@@ -2927,7 +2927,7 @@
     </row>
     <row r="105">
       <c r="A105" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
@@ -2935,13 +2935,13 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>5169.24</v>
+        <v>20331</v>
       </c>
       <c r="D105" t="n">
-        <v>5169.2357</v>
+        <v>20331.0046</v>
       </c>
       <c r="E105" t="n">
-        <v>-0.004299999999602733</v>
+        <v>0.004600000000209548</v>
       </c>
       <c r="F105" t="inlineStr">
         <is>
@@ -2951,7 +2951,7 @@
     </row>
     <row r="106">
       <c r="A106" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B106" t="inlineStr">
         <is>
@@ -2959,13 +2959,13 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>3200.94</v>
+        <v>8323.24</v>
       </c>
       <c r="D106" t="n">
-        <v>3200.936</v>
+        <v>8323.2374</v>
       </c>
       <c r="E106" t="n">
-        <v>-0.00400000000036016</v>
+        <v>-0.002599999999802094</v>
       </c>
       <c r="F106" t="inlineStr">
         <is>
@@ -2975,7 +2975,7 @@
     </row>
     <row r="107">
       <c r="A107" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
@@ -2983,13 +2983,13 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>4086.52</v>
+        <v>14156.74</v>
       </c>
       <c r="D107" t="n">
-        <v>4086.5203</v>
+        <v>14156.7402</v>
       </c>
       <c r="E107" t="n">
-        <v>0.0003000000001520675</v>
+        <v>0.0002000000004045432</v>
       </c>
       <c r="F107" t="inlineStr">
         <is>
@@ -2999,7 +2999,7 @@
     </row>
     <row r="108">
       <c r="A108" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
@@ -3007,13 +3007,13 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>3571.7</v>
+        <v>9639.219999999999</v>
       </c>
       <c r="D108" t="n">
-        <v>3571.6953</v>
+        <v>9639.2209</v>
       </c>
       <c r="E108" t="n">
-        <v>-0.004699999999957072</v>
+        <v>0.0009000000009109499</v>
       </c>
       <c r="F108" t="inlineStr">
         <is>
@@ -3023,7 +3023,7 @@
     </row>
     <row r="109">
       <c r="A109" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B109" t="inlineStr">
         <is>
@@ -3031,13 +3031,13 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>2909.35</v>
+        <v>4671.16</v>
       </c>
       <c r="D109" t="n">
-        <v>2909.3548</v>
+        <v>4671.1626</v>
       </c>
       <c r="E109" t="n">
-        <v>0.004800000000159343</v>
+        <v>0.002599999999802094</v>
       </c>
       <c r="F109" t="inlineStr">
         <is>
@@ -3047,7 +3047,7 @@
     </row>
     <row r="110">
       <c r="A110" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B110" t="inlineStr">
         <is>
@@ -3055,13 +3055,13 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>17537.06</v>
+        <v>17406.21</v>
       </c>
       <c r="D110" t="n">
-        <v>17537.0626</v>
+        <v>17406.2103</v>
       </c>
       <c r="E110" t="n">
-        <v>0.002599999999802094</v>
+        <v>0.0002999999996973202</v>
       </c>
       <c r="F110" t="inlineStr">
         <is>
@@ -3071,7 +3071,7 @@
     </row>
     <row r="111">
       <c r="A111" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B111" t="inlineStr">
         <is>
@@ -3079,13 +3079,13 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>1543.32</v>
+        <v>4695.52</v>
       </c>
       <c r="D111" t="n">
-        <v>1543.3212</v>
+        <v>4695.5248</v>
       </c>
       <c r="E111" t="n">
-        <v>0.001199999999926149</v>
+        <v>0.004799999999704596</v>
       </c>
       <c r="F111" t="inlineStr">
         <is>
@@ -3095,7 +3095,7 @@
     </row>
     <row r="112">
       <c r="A112" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B112" t="inlineStr">
         <is>
@@ -3103,13 +3103,13 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>6678.23</v>
+        <v>12436.8</v>
       </c>
       <c r="D112" t="n">
-        <v>6678.2308</v>
+        <v>12436.7979</v>
       </c>
       <c r="E112" t="n">
-        <v>0.0008000000007086783</v>
+        <v>-0.002099999999700231</v>
       </c>
       <c r="F112" t="inlineStr">
         <is>
@@ -3119,7 +3119,7 @@
     </row>
     <row r="113">
       <c r="A113" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B113" t="inlineStr">
         <is>
@@ -3127,13 +3127,13 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>3049.02</v>
+        <v>10177.44</v>
       </c>
       <c r="D113" t="n">
-        <v>3049.02</v>
+        <v>10177.4353</v>
       </c>
       <c r="E113" t="n">
-        <v>0</v>
+        <v>-0.004700000001321314</v>
       </c>
       <c r="F113" t="inlineStr">
         <is>
@@ -3143,7 +3143,7 @@
     </row>
     <row r="114">
       <c r="A114" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B114" t="inlineStr">
         <is>
@@ -3151,13 +3151,13 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>2511.93</v>
+        <v>6824.39</v>
       </c>
       <c r="D114" t="n">
-        <v>2511.9292</v>
+        <v>6824.3917</v>
       </c>
       <c r="E114" t="n">
-        <v>-0.0008000000002539309</v>
+        <v>0.001699999999800639</v>
       </c>
       <c r="F114" t="inlineStr">
         <is>
@@ -3167,7 +3167,7 @@
     </row>
     <row r="115">
       <c r="A115" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B115" t="inlineStr">
         <is>
@@ -3175,13 +3175,13 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>3529.07</v>
+        <v>15837.23</v>
       </c>
       <c r="D115" t="n">
-        <v>3529.0717</v>
+        <v>15837.2251</v>
       </c>
       <c r="E115" t="n">
-        <v>0.001699999999800639</v>
+        <v>-0.004899999999906868</v>
       </c>
       <c r="F115" t="inlineStr">
         <is>
@@ -3191,7 +3191,7 @@
     </row>
     <row r="116">
       <c r="A116" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B116" t="inlineStr">
         <is>
@@ -3199,13 +3199,13 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>8549.6</v>
+        <v>16147.61</v>
       </c>
       <c r="D116" t="n">
-        <v>8549.5996</v>
+        <v>16147.6051</v>
       </c>
       <c r="E116" t="n">
-        <v>-0.0004000000008090865</v>
+        <v>-0.004899999998087878</v>
       </c>
       <c r="F116" t="inlineStr">
         <is>
@@ -3215,7 +3215,7 @@
     </row>
     <row r="117">
       <c r="A117" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B117" t="inlineStr">
         <is>
@@ -3223,13 +3223,13 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>5057.58</v>
+        <v>6690.69</v>
       </c>
       <c r="D117" t="n">
-        <v>5057.5812</v>
+        <v>6690.685899999999</v>
       </c>
       <c r="E117" t="n">
-        <v>0.001199999999698775</v>
+        <v>-0.004100000000107684</v>
       </c>
       <c r="F117" t="inlineStr">
         <is>
@@ -3239,7 +3239,7 @@
     </row>
     <row r="118">
       <c r="A118" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B118" t="inlineStr">
         <is>
@@ -3247,13 +3247,13 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>4943.58</v>
+        <v>9293.190000000001</v>
       </c>
       <c r="D118" t="n">
-        <v>4943.5844</v>
+        <v>9293.189700000001</v>
       </c>
       <c r="E118" t="n">
-        <v>0.004399999999805004</v>
+        <v>-0.0002999999996973202</v>
       </c>
       <c r="F118" t="inlineStr">
         <is>
@@ -3263,7 +3263,7 @@
     </row>
     <row r="119">
       <c r="A119" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B119" t="inlineStr">
         <is>
@@ -3271,13 +3271,13 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>2695.31</v>
+        <v>6002.17</v>
       </c>
       <c r="D119" t="n">
-        <v>2695.3132</v>
+        <v>6002.1678</v>
       </c>
       <c r="E119" t="n">
-        <v>0.003200000000106229</v>
+        <v>-0.002199999999902502</v>
       </c>
       <c r="F119" t="inlineStr">
         <is>
@@ -3287,7 +3287,7 @@
     </row>
     <row r="120">
       <c r="A120" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B120" t="inlineStr">
         <is>
@@ -3295,13 +3295,13 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>3686.98</v>
+        <v>5946.19</v>
       </c>
       <c r="D120" t="n">
-        <v>3723.97</v>
+        <v>5951.6804</v>
       </c>
       <c r="E120" t="n">
-        <v>36.99000000000024</v>
+        <v>5.490400000000591</v>
       </c>
       <c r="F120" t="inlineStr">
         <is>
@@ -3311,7 +3311,7 @@
     </row>
     <row r="121">
       <c r="A121" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B121" t="inlineStr">
         <is>
@@ -3319,13 +3319,13 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>4134.09</v>
+        <v>4220.27</v>
       </c>
       <c r="D121" t="n">
-        <v>4134.0862</v>
+        <v>4220.266199999999</v>
       </c>
       <c r="E121" t="n">
-        <v>-0.003800000000410364</v>
+        <v>-0.003800000001319859</v>
       </c>
       <c r="F121" t="inlineStr">
         <is>
@@ -3335,7 +3335,7 @@
     </row>
     <row r="122">
       <c r="A122" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B122" t="inlineStr">
         <is>
@@ -3343,13 +3343,13 @@
         </is>
       </c>
       <c r="C122" t="n">
-        <v>10213.02</v>
+        <v>21175.44</v>
       </c>
       <c r="D122" t="n">
-        <v>10213.0191</v>
+        <v>21175.4425</v>
       </c>
       <c r="E122" t="n">
-        <v>-0.0008999999990919605</v>
+        <v>0.002500000002328306</v>
       </c>
       <c r="F122" t="inlineStr">
         <is>
@@ -3359,7 +3359,7 @@
     </row>
     <row r="123">
       <c r="A123" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B123" t="inlineStr">
         <is>
@@ -3367,13 +3367,13 @@
         </is>
       </c>
       <c r="C123" t="n">
-        <v>2947.25</v>
+        <v>8311.26</v>
       </c>
       <c r="D123" t="n">
-        <v>2947.2458</v>
+        <v>8311.262699999999</v>
       </c>
       <c r="E123" t="n">
-        <v>-0.004200000000309956</v>
+        <v>0.002699999999094871</v>
       </c>
       <c r="F123" t="inlineStr">
         <is>
@@ -3383,7 +3383,7 @@
     </row>
     <row r="124">
       <c r="A124" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B124" t="inlineStr">
         <is>
@@ -3391,13 +3391,13 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>5976.26</v>
+        <v>11339.94</v>
       </c>
       <c r="D124" t="n">
-        <v>5976.2576</v>
+        <v>11339.9365</v>
       </c>
       <c r="E124" t="n">
-        <v>-0.002400000000307045</v>
+        <v>-0.003500000000713044</v>
       </c>
       <c r="F124" t="inlineStr">
         <is>
@@ -3407,7 +3407,7 @@
     </row>
     <row r="125">
       <c r="A125" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B125" t="inlineStr">
         <is>
@@ -3415,13 +3415,13 @@
         </is>
       </c>
       <c r="C125" t="n">
-        <v>9032.299999999999</v>
+        <v>18638.3</v>
       </c>
       <c r="D125" t="n">
-        <v>9032.303599999999</v>
+        <v>18638.2999</v>
       </c>
       <c r="E125" t="n">
-        <v>0.003600000000005821</v>
+        <v>-0.0001000000011117663</v>
       </c>
       <c r="F125" t="inlineStr">
         <is>
@@ -3431,7 +3431,7 @@
     </row>
     <row r="126">
       <c r="A126" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B126" t="inlineStr">
         <is>
@@ -3439,13 +3439,13 @@
         </is>
       </c>
       <c r="C126" t="n">
-        <v>2970</v>
+        <v>0</v>
       </c>
       <c r="D126" t="n">
-        <v>5148</v>
+        <v>495</v>
       </c>
       <c r="E126" t="n">
-        <v>2178</v>
+        <v>495</v>
       </c>
       <c r="F126" t="inlineStr">
         <is>
@@ -3455,7 +3455,7 @@
     </row>
     <row r="127">
       <c r="A127" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B127" t="inlineStr">
         <is>
@@ -3463,13 +3463,13 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>16493.27</v>
+        <v>20031.02</v>
       </c>
       <c r="D127" t="n">
-        <v>16493.2711</v>
+        <v>20031.0245</v>
       </c>
       <c r="E127" t="n">
-        <v>0.001100000001315493</v>
+        <v>0.004499999999097781</v>
       </c>
       <c r="F127" t="inlineStr">
         <is>
@@ -3479,7 +3479,7 @@
     </row>
     <row r="128">
       <c r="A128" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B128" t="inlineStr">
         <is>
@@ -3487,13 +3487,13 @@
         </is>
       </c>
       <c r="C128" t="n">
-        <v>4399.85</v>
+        <v>11928.83</v>
       </c>
       <c r="D128" t="n">
-        <v>4399.8543</v>
+        <v>11928.8294</v>
       </c>
       <c r="E128" t="n">
-        <v>0.004299999999602733</v>
+        <v>-0.0005999999975756509</v>
       </c>
       <c r="F128" t="inlineStr">
         <is>
@@ -3503,7 +3503,7 @@
     </row>
     <row r="129">
       <c r="A129" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B129" t="inlineStr">
         <is>
@@ -3511,13 +3511,13 @@
         </is>
       </c>
       <c r="C129" t="n">
-        <v>4760.17</v>
+        <v>11059.52</v>
       </c>
       <c r="D129" t="n">
-        <v>4760.1697</v>
+        <v>11059.5231</v>
       </c>
       <c r="E129" t="n">
-        <v>-0.0002999999996973202</v>
+        <v>0.003099999999903957</v>
       </c>
       <c r="F129" t="inlineStr">
         <is>
@@ -3527,7 +3527,7 @@
     </row>
     <row r="130">
       <c r="A130" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B130" t="inlineStr">
         <is>
@@ -3535,13 +3535,13 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>4771.34</v>
+        <v>10955.82</v>
       </c>
       <c r="D130" t="n">
-        <v>4771.3378</v>
+        <v>10955.8194</v>
       </c>
       <c r="E130" t="n">
-        <v>-0.002199999999902502</v>
+        <v>-0.0005999999993946403</v>
       </c>
       <c r="F130" t="inlineStr">
         <is>
@@ -3551,7 +3551,7 @@
     </row>
     <row r="131">
       <c r="A131" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B131" t="inlineStr">
         <is>
@@ -3559,13 +3559,13 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>2862.32</v>
+        <v>8044.41</v>
       </c>
       <c r="D131" t="n">
-        <v>2862.3234</v>
+        <v>8044.411</v>
       </c>
       <c r="E131" t="n">
-        <v>0.003400000000056025</v>
+        <v>0.001000000000203727</v>
       </c>
       <c r="F131" t="inlineStr">
         <is>
@@ -3575,7 +3575,7 @@
     </row>
     <row r="132">
       <c r="A132" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B132" t="inlineStr">
         <is>
@@ -3583,13 +3583,13 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>6433.86</v>
+        <v>11135.26</v>
       </c>
       <c r="D132" t="n">
-        <v>6433.8627</v>
+        <v>11135.2562</v>
       </c>
       <c r="E132" t="n">
-        <v>0.002700000000004366</v>
+        <v>-0.003800000000410364</v>
       </c>
       <c r="F132" t="inlineStr">
         <is>
@@ -3599,7 +3599,7 @@
     </row>
     <row r="133">
       <c r="A133" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B133" t="inlineStr">
         <is>
@@ -3607,13 +3607,13 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>4022.7</v>
+        <v>11184.3</v>
       </c>
       <c r="D133" t="n">
-        <v>4022.7027</v>
+        <v>11184.3005</v>
       </c>
       <c r="E133" t="n">
-        <v>0.002700000000459113</v>
+        <v>0.000499999998282874</v>
       </c>
       <c r="F133" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     </row>
     <row r="134">
       <c r="A134" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B134" t="inlineStr">
         <is>
@@ -3631,13 +3631,13 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>3832.89</v>
+        <v>5732.65</v>
       </c>
       <c r="D134" t="n">
-        <v>3832.8892</v>
+        <v>5732.6539</v>
       </c>
       <c r="E134" t="n">
-        <v>-0.0008000000002539309</v>
+        <v>0.003900000000612636</v>
       </c>
       <c r="F134" t="inlineStr">
         <is>
@@ -3647,7 +3647,7 @@
     </row>
     <row r="135">
       <c r="A135" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B135" t="inlineStr">
         <is>
@@ -3655,13 +3655,13 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>2961.33</v>
+        <v>7254.76</v>
       </c>
       <c r="D135" t="n">
-        <v>2961.3328</v>
+        <v>7254.759100000001</v>
       </c>
       <c r="E135" t="n">
-        <v>0.00279999999975189</v>
+        <v>-0.0008999999990919605</v>
       </c>
       <c r="F135" t="inlineStr">
         <is>
@@ -3671,7 +3671,7 @@
     </row>
     <row r="136">
       <c r="A136" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B136" t="inlineStr">
         <is>
@@ -3679,13 +3679,13 @@
         </is>
       </c>
       <c r="C136" t="n">
-        <v>3489.06</v>
+        <v>4778.74</v>
       </c>
       <c r="D136" t="n">
-        <v>3489.06</v>
+        <v>4778.7433</v>
       </c>
       <c r="E136" t="n">
-        <v>0</v>
+        <v>0.003300000000308501</v>
       </c>
       <c r="F136" t="inlineStr">
         <is>
@@ -3695,7 +3695,7 @@
     </row>
     <row r="137">
       <c r="A137" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B137" t="inlineStr">
         <is>
@@ -3703,13 +3703,13 @@
         </is>
       </c>
       <c r="C137" t="n">
-        <v>4741.38</v>
+        <v>19123.83</v>
       </c>
       <c r="D137" t="n">
-        <v>4741.3778</v>
+        <v>19123.828</v>
       </c>
       <c r="E137" t="n">
-        <v>-0.002199999999902502</v>
+        <v>-0.002000000004045432</v>
       </c>
       <c r="F137" t="inlineStr">
         <is>
@@ -3719,7 +3719,7 @@
     </row>
     <row r="138">
       <c r="A138" s="1" t="n">
-        <v>46126</v>
+        <v>46122</v>
       </c>
       <c r="B138" t="inlineStr">
         <is>
@@ -3727,13 +3727,13 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>4810.83</v>
+        <v>14462.7</v>
       </c>
       <c r="D138" t="n">
-        <v>4810.825800000001</v>
+        <v>14462.6979</v>
       </c>
       <c r="E138" t="n">
-        <v>-0.004199999999400461</v>
+        <v>-0.002099999999700231</v>
       </c>
       <c r="F138" t="inlineStr">
         <is>
@@ -3774,7 +3774,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>133</v>
+        <v>129</v>
       </c>
     </row>
     <row r="3">
@@ -3784,7 +3784,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove outdated revenue data files and update Snowflake connection handling
- Deleted per_day_revenue.csv files and associated PDF reports to remove outdated revenue data.
- Updated the Snowflake connection logic in snowflake_client.py and sz_rev_valid_full.py to support optional role parameter.
- Modified Snowflake configuration to use new user and account details for production access.
- Removed parks_list.csv as it is no longer needed.
</commit_message>
<xml_diff>
--- a/data/output/revenue_comparison.xlsx
+++ b/data/output/revenue_comparison.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F138"/>
+  <dimension ref="A1:F139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -455,7 +455,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -466,10 +466,10 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>6962.8017</v>
+        <v>15397.638</v>
       </c>
       <c r="E2" t="n">
-        <v>6962.8017</v>
+        <v>15397.638</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -479,7 +479,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -487,13 +487,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>4895.49</v>
+        <v>6262.23</v>
       </c>
       <c r="D3" t="n">
-        <v>4895.49</v>
+        <v>6262.230000000001</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>1.818989403545856e-12</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -503,7 +503,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -511,13 +511,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1235.46</v>
+        <v>1227.6</v>
       </c>
       <c r="D4" t="n">
-        <v>1235.4622</v>
+        <v>1227.6026</v>
       </c>
       <c r="E4" t="n">
-        <v>0.002199999999902502</v>
+        <v>0.002600000000256841</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -527,7 +527,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -535,13 +535,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>2863.14</v>
+        <v>5356.66</v>
       </c>
       <c r="D5" t="n">
-        <v>2863.1435</v>
+        <v>5356.6575</v>
       </c>
       <c r="E5" t="n">
-        <v>0.003500000000258296</v>
+        <v>-0.002499999999599822</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -551,7 +551,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -559,13 +559,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>2029.27</v>
+        <v>2077.25</v>
       </c>
       <c r="D6" t="n">
-        <v>2029.2686</v>
+        <v>2077.2495</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.001400000000103319</v>
+        <v>-0.0004999999996471161</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -575,7 +575,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -583,13 +583,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>3842.72</v>
+        <v>5432.96</v>
       </c>
       <c r="D7" t="n">
-        <v>3842.724</v>
+        <v>5432.958000000001</v>
       </c>
       <c r="E7" t="n">
-        <v>0.00400000000036016</v>
+        <v>-0.001999999999497959</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -599,7 +599,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -607,13 +607,13 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>4812.03</v>
+        <v>11228.41</v>
       </c>
       <c r="D8" t="n">
-        <v>4812.0297</v>
+        <v>11228.4071</v>
       </c>
       <c r="E8" t="n">
-        <v>-0.0002999999996973202</v>
+        <v>-0.002899999999499414</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -623,7 +623,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -631,10 +631,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>43900</v>
+        <v>101132</v>
       </c>
       <c r="D9" t="n">
-        <v>43900</v>
+        <v>101132</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
@@ -647,7 +647,7 @@
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -655,13 +655,13 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>3713.63</v>
+        <v>9001.389999999999</v>
       </c>
       <c r="D10" t="n">
-        <v>3713.6334</v>
+        <v>9001.3871</v>
       </c>
       <c r="E10" t="n">
-        <v>0.003399999999601278</v>
+        <v>-0.002899999999499414</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -671,7 +671,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -679,23 +679,23 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>9306.809999999999</v>
+        <v>8831.540000000001</v>
       </c>
       <c r="D11" t="n">
-        <v>9306.811</v>
+        <v>8744.570900000001</v>
       </c>
       <c r="E11" t="n">
-        <v>0.001000000000203727</v>
+        <v>-86.96910000000025</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Match</t>
+          <t>Mismatch</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -703,13 +703,13 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>12122.84</v>
+        <v>22190.92</v>
       </c>
       <c r="D12" t="n">
-        <v>12122.8389</v>
+        <v>22190.9196</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.001100000001315493</v>
+        <v>-0.0003999999971711077</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -719,7 +719,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -727,13 +727,13 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>4040.07</v>
+        <v>4821.77</v>
       </c>
       <c r="D13" t="n">
-        <v>4040.0734</v>
+        <v>4821.7703</v>
       </c>
       <c r="E13" t="n">
-        <v>0.003400000000056025</v>
+        <v>0.0002999999996973202</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -743,7 +743,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -751,13 +751,13 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>18126.65</v>
+        <v>13557.26</v>
       </c>
       <c r="D14" t="n">
-        <v>18126.6545</v>
+        <v>13557.2598</v>
       </c>
       <c r="E14" t="n">
-        <v>0.004499999999097781</v>
+        <v>-0.0001999999985855538</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -767,7 +767,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -775,13 +775,13 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>5510.69</v>
+        <v>5846.17</v>
       </c>
       <c r="D15" t="n">
-        <v>5510.6858</v>
+        <v>5846.169699999999</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.004199999999400461</v>
+        <v>-0.0003000000006068149</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -791,7 +791,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -799,13 +799,13 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2609.72</v>
+        <v>6940.48</v>
       </c>
       <c r="D16" t="n">
-        <v>2609.7198</v>
+        <v>6940.4832</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.0001999999999497959</v>
+        <v>0.003200000000106229</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -815,7 +815,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -823,13 +823,13 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>5203.05</v>
+        <v>6031.14</v>
       </c>
       <c r="D17" t="n">
-        <v>5203.0522</v>
+        <v>6031.140200000001</v>
       </c>
       <c r="E17" t="n">
-        <v>0.002199999999902502</v>
+        <v>0.0002000000004045432</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -839,7 +839,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -847,13 +847,13 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>4411.59</v>
+        <v>8023.98</v>
       </c>
       <c r="D18" t="n">
-        <v>4411.5921</v>
+        <v>8023.983899999999</v>
       </c>
       <c r="E18" t="n">
-        <v>0.002099999999700231</v>
+        <v>0.003899999999703141</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -863,7 +863,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -871,13 +871,13 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>13837.58</v>
+        <v>18219.81</v>
       </c>
       <c r="D19" t="n">
-        <v>13837.5794</v>
+        <v>18219.8105</v>
       </c>
       <c r="E19" t="n">
-        <v>-0.0005999999993946403</v>
+        <v>0.000499999998282874</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -887,7 +887,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -895,13 +895,13 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>4460.64</v>
+        <v>5538.83</v>
       </c>
       <c r="D20" t="n">
-        <v>4460.637400000001</v>
+        <v>5538.8298</v>
       </c>
       <c r="E20" t="n">
-        <v>-0.002599999999802094</v>
+        <v>-0.0002000000004045432</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -911,7 +911,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -919,13 +919,13 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>6814.76</v>
+        <v>6902.86</v>
       </c>
       <c r="D21" t="n">
-        <v>6814.762600000001</v>
+        <v>6902.8643</v>
       </c>
       <c r="E21" t="n">
-        <v>0.002600000000711589</v>
+        <v>0.004300000000512227</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -935,7 +935,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -943,13 +943,13 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>3632.22</v>
+        <v>12659.65</v>
       </c>
       <c r="D22" t="n">
-        <v>3632.2241</v>
+        <v>12659.6504</v>
       </c>
       <c r="E22" t="n">
-        <v>0.004100000000107684</v>
+        <v>0.0004000000008090865</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -959,7 +959,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -967,13 +967,13 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>2583.83</v>
+        <v>7814.64</v>
       </c>
       <c r="D23" t="n">
-        <v>2583.8338</v>
+        <v>7814.6439</v>
       </c>
       <c r="E23" t="n">
-        <v>0.003799999999955617</v>
+        <v>0.003899999999703141</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -983,7 +983,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -991,13 +991,13 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>6469.53</v>
+        <v>7232.13</v>
       </c>
       <c r="D24" t="n">
-        <v>6469.531599999999</v>
+        <v>7232.1252</v>
       </c>
       <c r="E24" t="n">
-        <v>0.001599999999598367</v>
+        <v>-0.004799999999704596</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -1007,7 +1007,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -1015,23 +1015,23 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>4251.29</v>
+        <v>11933.12</v>
       </c>
       <c r="D25" t="n">
-        <v>4226.3</v>
+        <v>11933.1226</v>
       </c>
       <c r="E25" t="n">
-        <v>-24.98999999999978</v>
+        <v>0.002599999999802094</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Mismatch</t>
+          <t>Match</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -1039,13 +1039,13 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>4623.47</v>
+        <v>7526.34</v>
       </c>
       <c r="D26" t="n">
-        <v>4623.4701</v>
+        <v>7526.335899999999</v>
       </c>
       <c r="E26" t="n">
-        <v>9.999999929277692e-05</v>
+        <v>-0.004100000001017179</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -1055,7 +1055,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -1063,23 +1063,23 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>13883.06</v>
+        <v>11354.37</v>
       </c>
       <c r="D27" t="n">
-        <v>13883.0551</v>
+        <v>11354.365</v>
       </c>
       <c r="E27" t="n">
-        <v>-0.004899999998087878</v>
+        <v>-0.005000000002837623</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Match</t>
+          <t>Mismatch</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -1087,13 +1087,13 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>6836.81</v>
+        <v>13273.73</v>
       </c>
       <c r="D28" t="n">
-        <v>6836.810100000001</v>
+        <v>13273.7342</v>
       </c>
       <c r="E28" t="n">
-        <v>0.0001000000002022716</v>
+        <v>0.00420000000121945</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -1103,7 +1103,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -1111,13 +1111,13 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>6350.76</v>
+        <v>8148.24</v>
       </c>
       <c r="D29" t="n">
-        <v>6350.7634</v>
+        <v>8148.2373</v>
       </c>
       <c r="E29" t="n">
-        <v>0.003399999999601278</v>
+        <v>-0.002700000000004366</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -1127,7 +1127,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -1135,13 +1135,13 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>11408.23</v>
+        <v>11991.82</v>
       </c>
       <c r="D30" t="n">
-        <v>11408.233</v>
+        <v>11991.819</v>
       </c>
       <c r="E30" t="n">
-        <v>0.00300000000061118</v>
+        <v>-0.0009999999983847374</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -1151,7 +1151,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -1159,13 +1159,13 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>13632.59</v>
+        <v>18521.7</v>
       </c>
       <c r="D31" t="n">
-        <v>13632.5929</v>
+        <v>18521.7014</v>
       </c>
       <c r="E31" t="n">
-        <v>0.002899999999499414</v>
+        <v>0.001399999997374834</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -1175,7 +1175,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -1183,13 +1183,13 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>4067.21</v>
+        <v>10095.48</v>
       </c>
       <c r="D32" t="n">
-        <v>4067.2114</v>
+        <v>10095.4806</v>
       </c>
       <c r="E32" t="n">
-        <v>0.001400000000103319</v>
+        <v>0.0006000000012136297</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -1199,7 +1199,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -1207,13 +1207,13 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>8936.32</v>
+        <v>9269.33</v>
       </c>
       <c r="D33" t="n">
-        <v>8936.322699999999</v>
+        <v>9269.326300000001</v>
       </c>
       <c r="E33" t="n">
-        <v>0.002699999999094871</v>
+        <v>-0.003699999999298598</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -1223,7 +1223,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -1231,13 +1231,13 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>4408.47</v>
+        <v>8344.83</v>
       </c>
       <c r="D34" t="n">
-        <v>4408.4699</v>
+        <v>8344.827499999999</v>
       </c>
       <c r="E34" t="n">
-        <v>-0.0001000000002022716</v>
+        <v>-0.002500000000509317</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -1247,7 +1247,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -1255,13 +1255,13 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>2990.97</v>
+        <v>3625.43</v>
       </c>
       <c r="D35" t="n">
-        <v>2990.97</v>
+        <v>3625.43</v>
       </c>
       <c r="E35" t="n">
-        <v>4.547473508864641e-13</v>
+        <v>0</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -1271,7 +1271,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -1279,13 +1279,13 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>2895.38</v>
+        <v>7673.43</v>
       </c>
       <c r="D36" t="n">
-        <v>2895.3848</v>
+        <v>7673.4325</v>
       </c>
       <c r="E36" t="n">
-        <v>0.004800000000159343</v>
+        <v>0.002499999999599822</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -1295,7 +1295,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -1303,13 +1303,13 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>30646.34</v>
+        <v>18639.03</v>
       </c>
       <c r="D37" t="n">
-        <v>30646.3391</v>
+        <v>18639.0254</v>
       </c>
       <c r="E37" t="n">
-        <v>-0.0009000000027299393</v>
+        <v>-0.004599999996571569</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
@@ -1319,7 +1319,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -1327,13 +1327,13 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>8112.29</v>
+        <v>9844.59</v>
       </c>
       <c r="D38" t="n">
-        <v>8112.2859</v>
+        <v>9844.5929</v>
       </c>
       <c r="E38" t="n">
-        <v>-0.004100000000107684</v>
+        <v>0.002899999999499414</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
@@ -1343,7 +1343,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -1351,13 +1351,13 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>6864.92</v>
+        <v>8574.809999999999</v>
       </c>
       <c r="D39" t="n">
-        <v>6864.9221</v>
+        <v>8574.805999999999</v>
       </c>
       <c r="E39" t="n">
-        <v>0.002099999999700231</v>
+        <v>-0.004000000000814907</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
@@ -1367,7 +1367,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -1375,13 +1375,13 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>20669.13</v>
+        <v>18752.44</v>
       </c>
       <c r="D40" t="n">
-        <v>20669.1294</v>
+        <v>18752.4414</v>
       </c>
       <c r="E40" t="n">
-        <v>-0.0005999999993946403</v>
+        <v>0.001400000001012813</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
@@ -1391,7 +1391,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -1399,23 +1399,23 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>17580.33</v>
+        <v>20847.39</v>
       </c>
       <c r="D41" t="n">
-        <v>17580.3301</v>
+        <v>21397.3945</v>
       </c>
       <c r="E41" t="n">
-        <v>9.999999747378752e-05</v>
+        <v>550.0044999999991</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Match</t>
+          <t>Mismatch</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -1423,13 +1423,13 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>7644.91</v>
+        <v>6154.04</v>
       </c>
       <c r="D42" t="n">
-        <v>7644.9067</v>
+        <v>6154.035000000001</v>
       </c>
       <c r="E42" t="n">
-        <v>-0.003300000000308501</v>
+        <v>-0.004999999999199645</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
@@ -1439,7 +1439,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -1447,13 +1447,13 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>5514.33</v>
+        <v>7468.91</v>
       </c>
       <c r="D43" t="n">
-        <v>5514.3255</v>
+        <v>7468.9145</v>
       </c>
       <c r="E43" t="n">
-        <v>-0.004500000000007276</v>
+        <v>0.004500000000007276</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
@@ -1463,7 +1463,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -1471,13 +1471,13 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>9423.469999999999</v>
+        <v>10474.07</v>
       </c>
       <c r="D44" t="n">
-        <v>9423.4701</v>
+        <v>10474.0686</v>
       </c>
       <c r="E44" t="n">
-        <v>0.0001000000011117663</v>
+        <v>-0.001399999999193824</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
@@ -1487,7 +1487,7 @@
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -1495,13 +1495,13 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>4677.27</v>
+        <v>7397.7</v>
       </c>
       <c r="D45" t="n">
-        <v>4677.2734</v>
+        <v>7397.7003</v>
       </c>
       <c r="E45" t="n">
-        <v>0.003399999999601278</v>
+        <v>0.0002999999996973202</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
@@ -1511,7 +1511,7 @@
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
@@ -1519,13 +1519,13 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>3431.89</v>
+        <v>7800.79</v>
       </c>
       <c r="D46" t="n">
-        <v>3431.8897</v>
+        <v>7800.79</v>
       </c>
       <c r="E46" t="n">
-        <v>-0.0003000000001520675</v>
+        <v>0</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
@@ -1535,7 +1535,7 @@
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -1543,13 +1543,13 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>13101.72</v>
+        <v>10044.73</v>
       </c>
       <c r="D47" t="n">
-        <v>13101.7178</v>
+        <v>10044.7307</v>
       </c>
       <c r="E47" t="n">
-        <v>-0.002199999998993007</v>
+        <v>0.0007000000005064066</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
@@ -1559,7 +1559,7 @@
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
@@ -1567,13 +1567,13 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>4346.74</v>
+        <v>11740.32</v>
       </c>
       <c r="D48" t="n">
-        <v>4346.737599999999</v>
+        <v>11740.3234</v>
       </c>
       <c r="E48" t="n">
-        <v>-0.002400000000307045</v>
+        <v>0.003400000001420267</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
@@ -1583,7 +1583,7 @@
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
@@ -1591,13 +1591,13 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>12953.84</v>
+        <v>11292.67</v>
       </c>
       <c r="D49" t="n">
-        <v>12953.8394</v>
+        <v>11292.6653</v>
       </c>
       <c r="E49" t="n">
-        <v>-0.0006000000012136297</v>
+        <v>-0.004699999999502324</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
@@ -1607,7 +1607,7 @@
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
@@ -1615,13 +1615,13 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>9277.459999999999</v>
+        <v>8339.75</v>
       </c>
       <c r="D50" t="n">
-        <v>9277.455599999999</v>
+        <v>8339.7453</v>
       </c>
       <c r="E50" t="n">
-        <v>-0.004399999999805004</v>
+        <v>-0.004699999999502324</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
@@ -1631,7 +1631,7 @@
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
@@ -1639,13 +1639,13 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>5197.22</v>
+        <v>10591.57</v>
       </c>
       <c r="D51" t="n">
-        <v>5197.2196</v>
+        <v>10591.5691</v>
       </c>
       <c r="E51" t="n">
-        <v>-0.0003999999998995918</v>
+        <v>-0.0009000000009109499</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
@@ -1655,7 +1655,7 @@
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
@@ -1663,13 +1663,13 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>7848.93</v>
+        <v>7566.46</v>
       </c>
       <c r="D52" t="n">
-        <v>7848.928199999998</v>
+        <v>7566.455199999999</v>
       </c>
       <c r="E52" t="n">
-        <v>-0.0018000000018219</v>
+        <v>-0.004800000000614091</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
@@ -1679,7 +1679,7 @@
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
@@ -1687,13 +1687,13 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>2495.01</v>
+        <v>3729.2</v>
       </c>
       <c r="D53" t="n">
-        <v>2495.0053</v>
+        <v>3729.199</v>
       </c>
       <c r="E53" t="n">
-        <v>-0.004700000000411819</v>
+        <v>-0.001000000000203727</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
@@ -1703,7 +1703,7 @@
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
@@ -1711,13 +1711,13 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>6686.93</v>
+        <v>9792.559999999999</v>
       </c>
       <c r="D54" t="n">
-        <v>6686.933999999999</v>
+        <v>9792.558300000001</v>
       </c>
       <c r="E54" t="n">
-        <v>0.003999999998995918</v>
+        <v>-0.001699999998891144</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
@@ -1727,7 +1727,7 @@
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
@@ -1735,13 +1735,13 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>8344.24</v>
+        <v>14530.52</v>
       </c>
       <c r="D55" t="n">
-        <v>8344.239399999999</v>
+        <v>14530.5248</v>
       </c>
       <c r="E55" t="n">
-        <v>-0.0006000000012136297</v>
+        <v>0.004799999996976112</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
@@ -1751,45 +1751,45 @@
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>SKY ZONE HICKORY NC</t>
+          <t>SKY ZONE HAMPTON</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>11474.17</v>
+        <v>88</v>
       </c>
       <c r="D56" t="n">
-        <v>11474.17</v>
+        <v>0</v>
       </c>
       <c r="E56" t="n">
-        <v>-1.818989403545856e-12</v>
+        <v>-88</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Match</t>
+          <t>Mismatch</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>SKY ZONE HOUSTON COPPERFIELD TX</t>
+          <t>SKY ZONE HICKORY NC</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>970.77</v>
+        <v>11369.33</v>
       </c>
       <c r="D57" t="n">
-        <v>970.7706999999999</v>
+        <v>11369.3297</v>
       </c>
       <c r="E57" t="n">
-        <v>0.0006999999999379725</v>
+        <v>-0.000300000003335299</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
@@ -1799,69 +1799,69 @@
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>SKY ZONE HUNTINGTON BEACH CA</t>
+          <t>SKY ZONE HOUSTON COPPERFIELD TX</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>26273.91</v>
+        <v>5410.17</v>
       </c>
       <c r="D58" t="n">
-        <v>26364.527</v>
+        <v>5410.169</v>
       </c>
       <c r="E58" t="n">
-        <v>90.61700000000201</v>
+        <v>-0.001000000000203727</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Mismatch</t>
+          <t>Match</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>SKY ZONE KNOXVILLE</t>
+          <t>SKY ZONE HUNTINGTON BEACH CA</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>9975.18</v>
+        <v>27998.59</v>
       </c>
       <c r="D59" t="n">
-        <v>9975.180900000001</v>
+        <v>27922.6433</v>
       </c>
       <c r="E59" t="n">
-        <v>0.0009000000009109499</v>
+        <v>-75.94669999999678</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Match</t>
+          <t>Mismatch</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>SKY ZONE LAKELAND</t>
+          <t>SKY ZONE KNOXVILLE</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>6147.58</v>
+        <v>13653.53</v>
       </c>
       <c r="D60" t="n">
-        <v>6147.5838</v>
+        <v>13653.5349</v>
       </c>
       <c r="E60" t="n">
-        <v>0.003800000000410364</v>
+        <v>0.004899999999906868</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
@@ -1871,21 +1871,21 @@
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>SKY ZONE LANSING MI</t>
+          <t>SKY ZONE LAKELAND</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>3021.75</v>
+        <v>7479.25</v>
       </c>
       <c r="D61" t="n">
-        <v>3021.7542</v>
+        <v>7479.2532</v>
       </c>
       <c r="E61" t="n">
-        <v>0.004199999999855208</v>
+        <v>0.003200000000106229</v>
       </c>
       <c r="F61" t="inlineStr">
         <is>
@@ -1895,21 +1895,21 @@
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>SKY ZONE LITTLE ROCK AR</t>
+          <t>SKY ZONE LANSING MI</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>6322.5</v>
+        <v>4147.67</v>
       </c>
       <c r="D62" t="n">
-        <v>6322.501</v>
+        <v>4147.6732</v>
       </c>
       <c r="E62" t="n">
-        <v>0.001000000000203727</v>
+        <v>0.003200000000106229</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
@@ -1919,21 +1919,21 @@
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>SKY ZONE LOUISVILLE MIDDLETOWN</t>
+          <t>SKY ZONE LITTLE ROCK AR</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>14909.06</v>
+        <v>8363.08</v>
       </c>
       <c r="D63" t="n">
-        <v>14909.056</v>
+        <v>8363.077600000001</v>
       </c>
       <c r="E63" t="n">
-        <v>-0.003999999998995918</v>
+        <v>-0.002399999999397551</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
@@ -1943,21 +1943,21 @@
     </row>
     <row r="64">
       <c r="A64" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>SKY ZONE MANASSAS</t>
+          <t>SKY ZONE LOUISVILLE MIDDLETOWN</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>7145.87</v>
+        <v>11724.7</v>
       </c>
       <c r="D64" t="n">
-        <v>7145.874199999999</v>
+        <v>11724.7028</v>
       </c>
       <c r="E64" t="n">
-        <v>0.004199999999400461</v>
+        <v>0.002799999998387648</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
@@ -1967,21 +1967,21 @@
     </row>
     <row r="65">
       <c r="A65" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>SKY ZONE MAPLE GROVE</t>
+          <t>SKY ZONE MANASSAS</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>6021.58</v>
+        <v>8442.690000000001</v>
       </c>
       <c r="D65" t="n">
-        <v>6021.578299999999</v>
+        <v>8442.6913</v>
       </c>
       <c r="E65" t="n">
-        <v>-0.001700000000710133</v>
+        <v>0.001299999999901047</v>
       </c>
       <c r="F65" t="inlineStr">
         <is>
@@ -1991,21 +1991,21 @@
     </row>
     <row r="66">
       <c r="A66" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>SKY ZONE MAULDIN SC</t>
+          <t>SKY ZONE MAPLE GROVE</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>2765.61</v>
+        <v>6242.4</v>
       </c>
       <c r="D66" t="n">
-        <v>2765.6107</v>
+        <v>6242.403399999999</v>
       </c>
       <c r="E66" t="n">
-        <v>0.0007000000000516593</v>
+        <v>0.003399999999601278</v>
       </c>
       <c r="F66" t="inlineStr">
         <is>
@@ -2015,21 +2015,21 @@
     </row>
     <row r="67">
       <c r="A67" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>SKY ZONE MERCED</t>
+          <t>SKY ZONE MAULDIN SC</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>4946.34</v>
+        <v>6053.23</v>
       </c>
       <c r="D67" t="n">
-        <v>4946.3394</v>
+        <v>6053.2329</v>
       </c>
       <c r="E67" t="n">
-        <v>-0.000600000000304135</v>
+        <v>0.002900000000408909</v>
       </c>
       <c r="F67" t="inlineStr">
         <is>
@@ -2039,21 +2039,21 @@
     </row>
     <row r="68">
       <c r="A68" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>SKY ZONE METAIRIE</t>
+          <t>SKY ZONE MERCED</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>4502.54</v>
+        <v>5492.76</v>
       </c>
       <c r="D68" t="n">
-        <v>4502.5421</v>
+        <v>5492.7598</v>
       </c>
       <c r="E68" t="n">
-        <v>0.002099999999700231</v>
+        <v>-0.0002000000004045432</v>
       </c>
       <c r="F68" t="inlineStr">
         <is>
@@ -2063,21 +2063,21 @@
     </row>
     <row r="69">
       <c r="A69" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>SKY ZONE MISHAWAKA</t>
+          <t>SKY ZONE METAIRIE</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>14109.33</v>
+        <v>10025.97</v>
       </c>
       <c r="D69" t="n">
-        <v>14109.331</v>
+        <v>10025.9695</v>
       </c>
       <c r="E69" t="n">
-        <v>0.001000000000203727</v>
+        <v>-0.0005000000001018634</v>
       </c>
       <c r="F69" t="inlineStr">
         <is>
@@ -2087,21 +2087,21 @@
     </row>
     <row r="70">
       <c r="A70" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>SKY ZONE MISSION VIEJO</t>
+          <t>SKY ZONE MISHAWAKA</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>22093.13</v>
+        <v>10909.03</v>
       </c>
       <c r="D70" t="n">
-        <v>22093.1324</v>
+        <v>10909.0265</v>
       </c>
       <c r="E70" t="n">
-        <v>0.002399999997578561</v>
+        <v>-0.003500000002532033</v>
       </c>
       <c r="F70" t="inlineStr">
         <is>
@@ -2111,21 +2111,21 @@
     </row>
     <row r="71">
       <c r="A71" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>SKY ZONE MISSISSAUGA</t>
+          <t>SKY ZONE MISSION VIEJO</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>8694.700000000001</v>
+        <v>28612.01</v>
       </c>
       <c r="D71" t="n">
-        <v>8694.697900000001</v>
+        <v>28612.0094</v>
       </c>
       <c r="E71" t="n">
-        <v>-0.002099999999700231</v>
+        <v>-0.0006000000030326191</v>
       </c>
       <c r="F71" t="inlineStr">
         <is>
@@ -2135,21 +2135,21 @@
     </row>
     <row r="72">
       <c r="A72" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>SKY ZONE MODESTO</t>
+          <t>SKY ZONE MISSISSAUGA</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>9824.110000000001</v>
+        <v>12500.13</v>
       </c>
       <c r="D72" t="n">
-        <v>9824.107199999999</v>
+        <v>12500.1347</v>
       </c>
       <c r="E72" t="n">
-        <v>-0.002800000002025627</v>
+        <v>0.004699999999502324</v>
       </c>
       <c r="F72" t="inlineStr">
         <is>
@@ -2159,45 +2159,45 @@
     </row>
     <row r="73">
       <c r="A73" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>SKY ZONE MONROEVILLE PA</t>
+          <t>SKY ZONE MODESTO</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>3888.3</v>
+        <v>8888.469999999999</v>
       </c>
       <c r="D73" t="n">
-        <v>3840.32</v>
+        <v>8888.467799999999</v>
       </c>
       <c r="E73" t="n">
-        <v>-47.98000000000047</v>
+        <v>-0.002200000000811997</v>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Mismatch</t>
+          <t>Match</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>SKY ZONE MOUNT KISCO</t>
+          <t>SKY ZONE MONROEVILLE PA</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>6887.67</v>
+        <v>7336.53</v>
       </c>
       <c r="D74" t="n">
-        <v>6887.6705</v>
+        <v>7336.5318</v>
       </c>
       <c r="E74" t="n">
-        <v>0.0005000000001018634</v>
+        <v>0.00180000000000291</v>
       </c>
       <c r="F74" t="inlineStr">
         <is>
@@ -2207,69 +2207,69 @@
     </row>
     <row r="75">
       <c r="A75" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>SKY ZONE MOUNTLAKE TERRACE WA</t>
+          <t>SKY ZONE MOUNT KISCO</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>8967.540000000001</v>
+        <v>12630.97</v>
       </c>
       <c r="D75" t="n">
-        <v>8983.7212</v>
+        <v>12630.9745</v>
       </c>
       <c r="E75" t="n">
-        <v>16.18119999999908</v>
+        <v>0.004500000000916771</v>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Mismatch</t>
+          <t>Match</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>SKY ZONE MT OLIVE BUDD LAKE NJ</t>
+          <t>SKY ZONE MOUNTLAKE TERRACE WA</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>3968.6</v>
+        <v>12177.48</v>
       </c>
       <c r="D76" t="n">
-        <v>3968.5963</v>
+        <v>11664.062</v>
       </c>
       <c r="E76" t="n">
-        <v>-0.003700000000208092</v>
+        <v>-513.4179999999978</v>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Match</t>
+          <t>Mismatch</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>SKY ZONE MUSKEGON MI</t>
+          <t>SKY ZONE MT OLIVE BUDD LAKE NJ</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>2605.31</v>
+        <v>4732.14</v>
       </c>
       <c r="D77" t="n">
-        <v>2605.3118</v>
+        <v>4732.1355</v>
       </c>
       <c r="E77" t="n">
-        <v>0.00180000000000291</v>
+        <v>-0.004500000000007276</v>
       </c>
       <c r="F77" t="inlineStr">
         <is>
@@ -2279,21 +2279,21 @@
     </row>
     <row r="78">
       <c r="A78" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>SKY ZONE NAMPA ID</t>
+          <t>SKY ZONE MUSKEGON MI</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>7298.14</v>
+        <v>2082.68</v>
       </c>
       <c r="D78" t="n">
-        <v>7298.1446</v>
+        <v>2082.6822</v>
       </c>
       <c r="E78" t="n">
-        <v>0.004599999999300053</v>
+        <v>0.002199999999902502</v>
       </c>
       <c r="F78" t="inlineStr">
         <is>
@@ -2303,21 +2303,21 @@
     </row>
     <row r="79">
       <c r="A79" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>SKY ZONE NASHVILLE</t>
+          <t>SKY ZONE NAMPA ID</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>17555.06</v>
+        <v>5579.53</v>
       </c>
       <c r="D79" t="n">
-        <v>17555.0565</v>
+        <v>5579.528700000001</v>
       </c>
       <c r="E79" t="n">
-        <v>-0.003500000002532033</v>
+        <v>-0.001299999998991552</v>
       </c>
       <c r="F79" t="inlineStr">
         <is>
@@ -2327,21 +2327,21 @@
     </row>
     <row r="80">
       <c r="A80" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>SKY ZONE NEW ORLEANS</t>
+          <t>SKY ZONE NASHVILLE</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>9142.059999999999</v>
+        <v>19310.36</v>
       </c>
       <c r="D80" t="n">
-        <v>9142.060499999998</v>
+        <v>19310.3612</v>
       </c>
       <c r="E80" t="n">
-        <v>0.000499999998282874</v>
+        <v>0.001199999998789281</v>
       </c>
       <c r="F80" t="inlineStr">
         <is>
@@ -2351,21 +2351,21 @@
     </row>
     <row r="81">
       <c r="A81" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>SKY ZONE NEW ROCHELLE</t>
+          <t>SKY ZONE NEW ORLEANS</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>18063.83</v>
+        <v>10971.59</v>
       </c>
       <c r="D81" t="n">
-        <v>18063.8281</v>
+        <v>10971.5945</v>
       </c>
       <c r="E81" t="n">
-        <v>-0.001900000002933666</v>
+        <v>0.004500000000916771</v>
       </c>
       <c r="F81" t="inlineStr">
         <is>
@@ -2375,21 +2375,21 @@
     </row>
     <row r="82">
       <c r="A82" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>SKY ZONE NORTH FORT MYERS</t>
+          <t>SKY ZONE NEW ROCHELLE</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>7127.71</v>
+        <v>13075.02</v>
       </c>
       <c r="D82" t="n">
-        <v>7127.7131</v>
+        <v>13075.0238</v>
       </c>
       <c r="E82" t="n">
-        <v>0.003099999999903957</v>
+        <v>0.003799999998591375</v>
       </c>
       <c r="F82" t="inlineStr">
         <is>
@@ -2399,21 +2399,21 @@
     </row>
     <row r="83">
       <c r="A83" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>SKY ZONE NORTH INDIANAPOLIS</t>
+          <t>SKY ZONE NORTH FORT MYERS</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>7103.19</v>
+        <v>15862.95</v>
       </c>
       <c r="D83" t="n">
-        <v>7103.194599999999</v>
+        <v>15862.9513</v>
       </c>
       <c r="E83" t="n">
-        <v>0.004599999999300053</v>
+        <v>0.001299999999901047</v>
       </c>
       <c r="F83" t="inlineStr">
         <is>
@@ -2423,21 +2423,21 @@
     </row>
     <row r="84">
       <c r="A84" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>SKY ZONE OAKDALE</t>
+          <t>SKY ZONE NORTH INDIANAPOLIS</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>5081.59</v>
+        <v>12927.32</v>
       </c>
       <c r="D84" t="n">
-        <v>5081.5877</v>
+        <v>12927.3163</v>
       </c>
       <c r="E84" t="n">
-        <v>-0.002300000000104774</v>
+        <v>-0.003699999999298598</v>
       </c>
       <c r="F84" t="inlineStr">
         <is>
@@ -2447,21 +2447,21 @@
     </row>
     <row r="85">
       <c r="A85" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>SKY ZONE OAKS PHOENIXVILLE</t>
+          <t>SKY ZONE OAKDALE</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>2496.33</v>
+        <v>5829.85</v>
       </c>
       <c r="D85" t="n">
-        <v>2496.3317</v>
+        <v>5829.8451</v>
       </c>
       <c r="E85" t="n">
-        <v>0.001699999999800639</v>
+        <v>-0.004899999999906868</v>
       </c>
       <c r="F85" t="inlineStr">
         <is>
@@ -2471,21 +2471,21 @@
     </row>
     <row r="86">
       <c r="A86" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>SKY ZONE OCEAN</t>
+          <t>SKY ZONE OAKS PHOENIXVILLE</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>10024.15</v>
+        <v>7066.1</v>
       </c>
       <c r="D86" t="n">
-        <v>10024.1469</v>
+        <v>7066.102499999999</v>
       </c>
       <c r="E86" t="n">
-        <v>-0.003099999998084968</v>
+        <v>0.002499999998690328</v>
       </c>
       <c r="F86" t="inlineStr">
         <is>
@@ -2495,21 +2495,21 @@
     </row>
     <row r="87">
       <c r="A87" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>SKY ZONE OLYMPIA</t>
+          <t>SKY ZONE OCEAN</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>13086.02</v>
+        <v>11942.5</v>
       </c>
       <c r="D87" t="n">
-        <v>13086.0181</v>
+        <v>11942.4959</v>
       </c>
       <c r="E87" t="n">
-        <v>-0.001900000001114677</v>
+        <v>-0.004100000000107684</v>
       </c>
       <c r="F87" t="inlineStr">
         <is>
@@ -2519,21 +2519,21 @@
     </row>
     <row r="88">
       <c r="A88" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>SKY ZONE ORLAND PARK</t>
+          <t>SKY ZONE OLYMPIA</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>10428.66</v>
+        <v>12617.54</v>
       </c>
       <c r="D88" t="n">
-        <v>10428.6631</v>
+        <v>12617.5421</v>
       </c>
       <c r="E88" t="n">
-        <v>0.003099999998084968</v>
+        <v>0.002099999999700231</v>
       </c>
       <c r="F88" t="inlineStr">
         <is>
@@ -2543,21 +2543,21 @@
     </row>
     <row r="89">
       <c r="A89" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>SKY ZONE ORLANDO</t>
+          <t>SKY ZONE ORLAND PARK</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>6938.56</v>
+        <v>10976.23</v>
       </c>
       <c r="D89" t="n">
-        <v>6938.557000000001</v>
+        <v>10976.2314</v>
       </c>
       <c r="E89" t="n">
-        <v>-0.002999999999701686</v>
+        <v>0.001399999999193824</v>
       </c>
       <c r="F89" t="inlineStr">
         <is>
@@ -2567,21 +2567,21 @@
     </row>
     <row r="90">
       <c r="A90" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>SKY ZONE PALM BAY MELBOURNE FL</t>
+          <t>SKY ZONE ORLANDO</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>6221.92</v>
+        <v>14384.01</v>
       </c>
       <c r="D90" t="n">
-        <v>6221.9221</v>
+        <v>14384.0059</v>
       </c>
       <c r="E90" t="n">
-        <v>0.002099999999700231</v>
+        <v>-0.004100000000107684</v>
       </c>
       <c r="F90" t="inlineStr">
         <is>
@@ -2591,21 +2591,21 @@
     </row>
     <row r="91">
       <c r="A91" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>SKY ZONE PALM SPRINGS</t>
+          <t>SKY ZONE PALM BAY MELBOURNE FL</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>5526.81</v>
+        <v>10399.24</v>
       </c>
       <c r="D91" t="n">
-        <v>5526.805799999999</v>
+        <v>10399.2395</v>
       </c>
       <c r="E91" t="n">
-        <v>-0.00420000000121945</v>
+        <v>-0.0005000000001018634</v>
       </c>
       <c r="F91" t="inlineStr">
         <is>
@@ -2615,21 +2615,21 @@
     </row>
     <row r="92">
       <c r="A92" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>SKY ZONE PARKER</t>
+          <t>SKY ZONE PALM SPRINGS</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>5940.29</v>
+        <v>19198.33</v>
       </c>
       <c r="D92" t="n">
-        <v>5940.2898</v>
+        <v>19198.33229999999</v>
       </c>
       <c r="E92" t="n">
-        <v>-0.0001999999994950485</v>
+        <v>0.002299999992828816</v>
       </c>
       <c r="F92" t="inlineStr">
         <is>
@@ -2639,21 +2639,21 @@
     </row>
     <row r="93">
       <c r="A93" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>SKY ZONE PENSACOLA</t>
+          <t>SKY ZONE PARKER</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>3998.32</v>
+        <v>6321.62</v>
       </c>
       <c r="D93" t="n">
-        <v>3998.3208</v>
+        <v>6321.617999999999</v>
       </c>
       <c r="E93" t="n">
-        <v>0.0007999999997991836</v>
+        <v>-0.002000000000407454</v>
       </c>
       <c r="F93" t="inlineStr">
         <is>
@@ -2663,45 +2663,45 @@
     </row>
     <row r="94">
       <c r="A94" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>SKY ZONE PEORIA AZ</t>
+          <t>SKY ZONE PENSACOLA</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>4822.33</v>
+        <v>6208.5</v>
       </c>
       <c r="D94" t="n">
-        <v>4822.3259</v>
+        <v>6208.495</v>
       </c>
       <c r="E94" t="n">
-        <v>-0.004100000000107684</v>
+        <v>-0.005000000000109139</v>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Match</t>
+          <t>Mismatch</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>SKY ZONE PHOENIX AZ</t>
+          <t>SKY ZONE PEORIA AZ</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>2073.83</v>
+        <v>7285.25</v>
       </c>
       <c r="D95" t="n">
-        <v>2073.8291</v>
+        <v>7285.2464</v>
       </c>
       <c r="E95" t="n">
-        <v>-0.0009000000000014552</v>
+        <v>-0.003600000000005821</v>
       </c>
       <c r="F95" t="inlineStr">
         <is>
@@ -2711,21 +2711,21 @@
     </row>
     <row r="96">
       <c r="A96" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>SKY ZONE PORT SAINT LUCIE FL</t>
+          <t>SKY ZONE PHOENIX AZ</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>6893.56</v>
+        <v>6584.59</v>
       </c>
       <c r="D96" t="n">
-        <v>6893.561899999999</v>
+        <v>6584.594899999999</v>
       </c>
       <c r="E96" t="n">
-        <v>0.001899999998386193</v>
+        <v>0.004899999998997373</v>
       </c>
       <c r="F96" t="inlineStr">
         <is>
@@ -2735,21 +2735,21 @@
     </row>
     <row r="97">
       <c r="A97" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>SKY ZONE PROVIDENCE RI</t>
+          <t>SKY ZONE PORT SAINT LUCIE FL</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>2036.77</v>
+        <v>10318.45</v>
       </c>
       <c r="D97" t="n">
-        <v>2036.7718</v>
+        <v>10318.4546</v>
       </c>
       <c r="E97" t="n">
-        <v>0.00180000000000291</v>
+        <v>0.004600000000209548</v>
       </c>
       <c r="F97" t="inlineStr">
         <is>
@@ -2759,69 +2759,69 @@
     </row>
     <row r="98">
       <c r="A98" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>SKY ZONE RANCHO CUCAMONGA</t>
+          <t>SKY ZONE PROVIDENCE RI</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>13449.81</v>
+        <v>4613.63</v>
       </c>
       <c r="D98" t="n">
-        <v>13544.7547</v>
+        <v>4613.6345</v>
       </c>
       <c r="E98" t="n">
-        <v>94.94470000000001</v>
+        <v>0.004500000000007276</v>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>Mismatch</t>
+          <t>Match</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>SKY ZONE RIVERSIDE</t>
+          <t>SKY ZONE RANCHO CUCAMONGA</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>8050.28</v>
+        <v>19538.42</v>
       </c>
       <c r="D99" t="n">
-        <v>8050.2823</v>
+        <v>19552.2577</v>
       </c>
       <c r="E99" t="n">
-        <v>0.002300000000104774</v>
+        <v>13.83770000000004</v>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>Match</t>
+          <t>Mismatch</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>SKY ZONE ROANOKE VA</t>
+          <t>SKY ZONE RIVERSIDE</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>3048.9</v>
+        <v>11179.42</v>
       </c>
       <c r="D100" t="n">
-        <v>3048.9047</v>
+        <v>11179.4172</v>
       </c>
       <c r="E100" t="n">
-        <v>0.004699999999502324</v>
+        <v>-0.002800000000206637</v>
       </c>
       <c r="F100" t="inlineStr">
         <is>
@@ -2831,21 +2831,21 @@
     </row>
     <row r="101">
       <c r="A101" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>SKY ZONE ROGERS AR</t>
+          <t>SKY ZONE ROANOKE VA</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>7216.29</v>
+        <v>5316.6</v>
       </c>
       <c r="D101" t="n">
-        <v>7216.2873</v>
+        <v>5316.5999</v>
       </c>
       <c r="E101" t="n">
-        <v>-0.002700000000004366</v>
+        <v>-0.0001000000002022716</v>
       </c>
       <c r="F101" t="inlineStr">
         <is>
@@ -2855,21 +2855,21 @@
     </row>
     <row r="102">
       <c r="A102" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>SKY ZONE ROSEVILLE</t>
+          <t>SKY ZONE ROGERS AR</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>12992.68</v>
+        <v>7713.67</v>
       </c>
       <c r="D102" t="n">
-        <v>12992.678</v>
+        <v>7713.673100000001</v>
       </c>
       <c r="E102" t="n">
-        <v>-0.002000000002226443</v>
+        <v>0.003100000000813452</v>
       </c>
       <c r="F102" t="inlineStr">
         <is>
@@ -2879,21 +2879,21 @@
     </row>
     <row r="103">
       <c r="A103" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>SKY ZONE ROSWELL GA</t>
+          <t>SKY ZONE ROSEVILLE</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>10464.08</v>
+        <v>13001.89</v>
       </c>
       <c r="D103" t="n">
-        <v>10464.0804</v>
+        <v>13001.8882</v>
       </c>
       <c r="E103" t="n">
-        <v>0.0004000000008090865</v>
+        <v>-0.00180000000000291</v>
       </c>
       <c r="F103" t="inlineStr">
         <is>
@@ -2903,21 +2903,21 @@
     </row>
     <row r="104">
       <c r="A104" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>SKY ZONE SACRAMENTO</t>
+          <t>SKY ZONE ROSWELL GA</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>11346.58</v>
+        <v>9084.040000000001</v>
       </c>
       <c r="D104" t="n">
-        <v>11346.5825</v>
+        <v>9084.042699999998</v>
       </c>
       <c r="E104" t="n">
-        <v>0.002500000000509317</v>
+        <v>0.002699999997275881</v>
       </c>
       <c r="F104" t="inlineStr">
         <is>
@@ -2927,21 +2927,21 @@
     </row>
     <row r="105">
       <c r="A105" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>SKY ZONE SAN CARLOS</t>
+          <t>SKY ZONE SACRAMENTO</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>20331</v>
+        <v>13354.85</v>
       </c>
       <c r="D105" t="n">
-        <v>20331.0046</v>
+        <v>13354.8451</v>
       </c>
       <c r="E105" t="n">
-        <v>0.004600000000209548</v>
+        <v>-0.004900000001725857</v>
       </c>
       <c r="F105" t="inlineStr">
         <is>
@@ -2951,21 +2951,21 @@
     </row>
     <row r="106">
       <c r="A106" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>SKY ZONE SAN JOSE</t>
+          <t>SKY ZONE SAN CARLOS</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>8323.24</v>
+        <v>21717.87</v>
       </c>
       <c r="D106" t="n">
-        <v>8323.2374</v>
+        <v>21717.8685</v>
       </c>
       <c r="E106" t="n">
-        <v>-0.002599999999802094</v>
+        <v>-0.00150000000212458</v>
       </c>
       <c r="F106" t="inlineStr">
         <is>
@@ -2975,21 +2975,21 @@
     </row>
     <row r="107">
       <c r="A107" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>SKY ZONE SANTA CLARITA CA</t>
+          <t>SKY ZONE SAN JOSE</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>14156.74</v>
+        <v>10232.21</v>
       </c>
       <c r="D107" t="n">
-        <v>14156.7402</v>
+        <v>10232.2117</v>
       </c>
       <c r="E107" t="n">
-        <v>0.0002000000004045432</v>
+        <v>0.001700000002529123</v>
       </c>
       <c r="F107" t="inlineStr">
         <is>
@@ -2999,21 +2999,21 @@
     </row>
     <row r="108">
       <c r="A108" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>SKY ZONE SAVANNAH GA</t>
+          <t>SKY ZONE SANTA CLARITA CA</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>9639.219999999999</v>
+        <v>14401.68</v>
       </c>
       <c r="D108" t="n">
-        <v>9639.2209</v>
+        <v>14401.6766</v>
       </c>
       <c r="E108" t="n">
-        <v>0.0009000000009109499</v>
+        <v>-0.003399999999601278</v>
       </c>
       <c r="F108" t="inlineStr">
         <is>
@@ -3023,21 +3023,21 @@
     </row>
     <row r="109">
       <c r="A109" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>SKY ZONE SCOTTSDALE AZ</t>
+          <t>SKY ZONE SAVANNAH GA</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>4671.16</v>
+        <v>14926.41</v>
       </c>
       <c r="D109" t="n">
-        <v>4671.1626</v>
+        <v>14926.4121</v>
       </c>
       <c r="E109" t="n">
-        <v>0.002599999999802094</v>
+        <v>0.00210000000151922</v>
       </c>
       <c r="F109" t="inlineStr">
         <is>
@@ -3047,21 +3047,21 @@
     </row>
     <row r="110">
       <c r="A110" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>SKY ZONE SEATTLE TUKWILA</t>
+          <t>SKY ZONE SCOTTSDALE AZ</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>17406.21</v>
+        <v>10016.5</v>
       </c>
       <c r="D110" t="n">
-        <v>17406.2103</v>
+        <v>10016.4985</v>
       </c>
       <c r="E110" t="n">
-        <v>0.0002999999996973202</v>
+        <v>-0.00150000000030559</v>
       </c>
       <c r="F110" t="inlineStr">
         <is>
@@ -3071,21 +3071,21 @@
     </row>
     <row r="111">
       <c r="A111" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>SKY ZONE SHORT PUMP</t>
+          <t>SKY ZONE SEATTLE TUKWILA</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>4695.52</v>
+        <v>21806.38</v>
       </c>
       <c r="D111" t="n">
-        <v>4695.5248</v>
+        <v>21806.3785</v>
       </c>
       <c r="E111" t="n">
-        <v>0.004799999999704596</v>
+        <v>-0.00150000000212458</v>
       </c>
       <c r="F111" t="inlineStr">
         <is>
@@ -3095,21 +3095,21 @@
     </row>
     <row r="112">
       <c r="A112" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>SKY ZONE SILVERDALE</t>
+          <t>SKY ZONE SHORT PUMP</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>12436.8</v>
+        <v>7012.18</v>
       </c>
       <c r="D112" t="n">
-        <v>12436.7979</v>
+        <v>7012.184799999999</v>
       </c>
       <c r="E112" t="n">
-        <v>-0.002099999999700231</v>
+        <v>0.004799999998795101</v>
       </c>
       <c r="F112" t="inlineStr">
         <is>
@@ -3119,21 +3119,21 @@
     </row>
     <row r="113">
       <c r="A113" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>SKY ZONE SOUTH PLAINFIELD PISCATAWAY NJ</t>
+          <t>SKY ZONE SILVERDALE</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>10177.44</v>
+        <v>8769.809999999999</v>
       </c>
       <c r="D113" t="n">
-        <v>10177.4353</v>
+        <v>8769.812900000001</v>
       </c>
       <c r="E113" t="n">
-        <v>-0.004700000001321314</v>
+        <v>0.002900000001318404</v>
       </c>
       <c r="F113" t="inlineStr">
         <is>
@@ -3143,21 +3143,21 @@
     </row>
     <row r="114">
       <c r="A114" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>SKY ZONE SPRING VALLEY NANUET NY</t>
+          <t>SKY ZONE SOUTH PLAINFIELD PISCATAWAY NJ</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>6824.39</v>
+        <v>7884.66</v>
       </c>
       <c r="D114" t="n">
-        <v>6824.3917</v>
+        <v>7884.659499999999</v>
       </c>
       <c r="E114" t="n">
-        <v>0.001699999999800639</v>
+        <v>-0.0005000000010113581</v>
       </c>
       <c r="F114" t="inlineStr">
         <is>
@@ -3167,21 +3167,21 @@
     </row>
     <row r="115">
       <c r="A115" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>SKY ZONE SPRINGFIELD NJ</t>
+          <t>SKY ZONE SPRING VALLEY NANUET NY</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>15837.23</v>
+        <v>8774.799999999999</v>
       </c>
       <c r="D115" t="n">
-        <v>15837.2251</v>
+        <v>8774.799999999999</v>
       </c>
       <c r="E115" t="n">
-        <v>-0.004899999999906868</v>
+        <v>0</v>
       </c>
       <c r="F115" t="inlineStr">
         <is>
@@ -3191,21 +3191,21 @@
     </row>
     <row r="116">
       <c r="A116" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>SKY ZONE SPRINGFIELD VA</t>
+          <t>SKY ZONE SPRINGFIELD NJ</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>16147.61</v>
+        <v>19324.57</v>
       </c>
       <c r="D116" t="n">
-        <v>16147.6051</v>
+        <v>19324.56689999999</v>
       </c>
       <c r="E116" t="n">
-        <v>-0.004899999998087878</v>
+        <v>-0.003100000005360926</v>
       </c>
       <c r="F116" t="inlineStr">
         <is>
@@ -3215,21 +3215,21 @@
     </row>
     <row r="117">
       <c r="A117" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>SKY ZONE SUMMERLIN LAS VEGAS</t>
+          <t>SKY ZONE SPRINGFIELD VA</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>6690.69</v>
+        <v>23931.28</v>
       </c>
       <c r="D117" t="n">
-        <v>6690.685899999999</v>
+        <v>23931.2801</v>
       </c>
       <c r="E117" t="n">
-        <v>-0.004100000000107684</v>
+        <v>9.999999747378752e-05</v>
       </c>
       <c r="F117" t="inlineStr">
         <is>
@@ -3239,21 +3239,21 @@
     </row>
     <row r="118">
       <c r="A118" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>SKY ZONE TACOMA WA</t>
+          <t>SKY ZONE SUMMERLIN LAS VEGAS</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>9293.190000000001</v>
+        <v>10937.28</v>
       </c>
       <c r="D118" t="n">
-        <v>9293.189700000001</v>
+        <v>10937.2782</v>
       </c>
       <c r="E118" t="n">
-        <v>-0.0002999999996973202</v>
+        <v>-0.00180000000000291</v>
       </c>
       <c r="F118" t="inlineStr">
         <is>
@@ -3263,21 +3263,21 @@
     </row>
     <row r="119">
       <c r="A119" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>SKY ZONE TAMPA</t>
+          <t>SKY ZONE TACOMA WA</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>6002.17</v>
+        <v>6948.89</v>
       </c>
       <c r="D119" t="n">
-        <v>6002.1678</v>
+        <v>6948.885199999999</v>
       </c>
       <c r="E119" t="n">
-        <v>-0.002199999999902502</v>
+        <v>-0.004800000001523586</v>
       </c>
       <c r="F119" t="inlineStr">
         <is>
@@ -3287,69 +3287,69 @@
     </row>
     <row r="120">
       <c r="A120" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>SKY ZONE TEMECULA</t>
+          <t>SKY ZONE TAMPA</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>5946.19</v>
+        <v>10464.4</v>
       </c>
       <c r="D120" t="n">
-        <v>5951.6804</v>
+        <v>10464.4001</v>
       </c>
       <c r="E120" t="n">
-        <v>5.490400000000591</v>
+        <v>9.999999929277692e-05</v>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>Mismatch</t>
+          <t>Match</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>SKY ZONE THORNTON</t>
+          <t>SKY ZONE TEMECULA</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>4220.27</v>
+        <v>10717.84</v>
       </c>
       <c r="D121" t="n">
-        <v>4220.266199999999</v>
+        <v>10608.2552</v>
       </c>
       <c r="E121" t="n">
-        <v>-0.003800000001319859</v>
+        <v>-109.5847999999987</v>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>Match</t>
+          <t>Mismatch</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>SKY ZONE THOUSAND OAKS</t>
+          <t>SKY ZONE THORNTON</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>21175.44</v>
+        <v>9250.610000000001</v>
       </c>
       <c r="D122" t="n">
-        <v>21175.4425</v>
+        <v>9250.6083</v>
       </c>
       <c r="E122" t="n">
-        <v>0.002500000002328306</v>
+        <v>-0.001700000000710133</v>
       </c>
       <c r="F122" t="inlineStr">
         <is>
@@ -3359,21 +3359,21 @@
     </row>
     <row r="123">
       <c r="A123" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>SKY ZONE TOLEDO HOLLAND</t>
+          <t>SKY ZONE THOUSAND OAKS</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>8311.26</v>
+        <v>23451.61</v>
       </c>
       <c r="D123" t="n">
-        <v>8311.262699999999</v>
+        <v>23451.6113</v>
       </c>
       <c r="E123" t="n">
-        <v>0.002699999999094871</v>
+        <v>0.001299999999901047</v>
       </c>
       <c r="F123" t="inlineStr">
         <is>
@@ -3383,21 +3383,21 @@
     </row>
     <row r="124">
       <c r="A124" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>SKY ZONE TORONTO</t>
+          <t>SKY ZONE TOLEDO HOLLAND</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>11339.94</v>
+        <v>8781.82</v>
       </c>
       <c r="D124" t="n">
-        <v>11339.9365</v>
+        <v>8781.8205</v>
       </c>
       <c r="E124" t="n">
-        <v>-0.003500000000713044</v>
+        <v>0.0005000000001018634</v>
       </c>
       <c r="F124" t="inlineStr">
         <is>
@@ -3407,21 +3407,21 @@
     </row>
     <row r="125">
       <c r="A125" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>SKY ZONE TORRANCE</t>
+          <t>SKY ZONE TORONTO</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>18638.3</v>
+        <v>18597.01</v>
       </c>
       <c r="D125" t="n">
-        <v>18638.2999</v>
+        <v>18597.0111</v>
       </c>
       <c r="E125" t="n">
-        <v>-0.0001000000011117663</v>
+        <v>0.001100000004953472</v>
       </c>
       <c r="F125" t="inlineStr">
         <is>
@@ -3431,69 +3431,69 @@
     </row>
     <row r="126">
       <c r="A126" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>SKY ZONE VALLEJO CA</t>
+          <t>SKY ZONE TORRANCE</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>0</v>
+        <v>23572.32</v>
       </c>
       <c r="D126" t="n">
-        <v>495</v>
+        <v>23572.3234</v>
       </c>
       <c r="E126" t="n">
-        <v>495</v>
+        <v>0.003400000001420267</v>
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>Mismatch</t>
+          <t>Match</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>SKY ZONE VAN NUYS CA</t>
+          <t>SKY ZONE VALLEJO CA</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>20031.02</v>
+        <v>18698.24</v>
       </c>
       <c r="D127" t="n">
-        <v>20031.0245</v>
+        <v>18857.4756</v>
       </c>
       <c r="E127" t="n">
-        <v>0.004499999999097781</v>
+        <v>159.2356</v>
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>Match</t>
+          <t>Mismatch</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>SKY ZONE VANCOUVER</t>
+          <t>SKY ZONE VAN NUYS CA</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>11928.83</v>
+        <v>31024.26</v>
       </c>
       <c r="D128" t="n">
-        <v>11928.8294</v>
+        <v>31024.2563</v>
       </c>
       <c r="E128" t="n">
-        <v>-0.0005999999975756509</v>
+        <v>-0.003699999997479608</v>
       </c>
       <c r="F128" t="inlineStr">
         <is>
@@ -3503,21 +3503,21 @@
     </row>
     <row r="129">
       <c r="A129" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>SKY ZONE VAUGHAN</t>
+          <t>SKY ZONE VANCOUVER</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>11059.52</v>
+        <v>10284.82</v>
       </c>
       <c r="D129" t="n">
-        <v>11059.5231</v>
+        <v>10284.8162</v>
       </c>
       <c r="E129" t="n">
-        <v>0.003099999999903957</v>
+        <v>-0.003799999998591375</v>
       </c>
       <c r="F129" t="inlineStr">
         <is>
@@ -3527,21 +3527,21 @@
     </row>
     <row r="130">
       <c r="A130" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>SKY ZONE VERNON HILLS</t>
+          <t>SKY ZONE VAUGHAN</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>10955.82</v>
+        <v>16589.1</v>
       </c>
       <c r="D130" t="n">
-        <v>10955.8194</v>
+        <v>16589.1029</v>
       </c>
       <c r="E130" t="n">
-        <v>-0.0005999999993946403</v>
+        <v>0.002900000003137393</v>
       </c>
       <c r="F130" t="inlineStr">
         <is>
@@ -3551,21 +3551,21 @@
     </row>
     <row r="131">
       <c r="A131" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>SKY ZONE VESTAL BINGHAMTON NY</t>
+          <t>SKY ZONE VERNON HILLS</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>8044.41</v>
+        <v>19463.67</v>
       </c>
       <c r="D131" t="n">
-        <v>8044.411</v>
+        <v>19463.6746</v>
       </c>
       <c r="E131" t="n">
-        <v>0.001000000000203727</v>
+        <v>0.004600000003847526</v>
       </c>
       <c r="F131" t="inlineStr">
         <is>
@@ -3575,21 +3575,21 @@
     </row>
     <row r="132">
       <c r="A132" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>SKY ZONE VISALIA</t>
+          <t>SKY ZONE VESTAL BINGHAMTON NY</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>11135.26</v>
+        <v>8137.73</v>
       </c>
       <c r="D132" t="n">
-        <v>11135.2562</v>
+        <v>8137.7264</v>
       </c>
       <c r="E132" t="n">
-        <v>-0.003800000000410364</v>
+        <v>-0.003599999999096326</v>
       </c>
       <c r="F132" t="inlineStr">
         <is>
@@ -3599,21 +3599,21 @@
     </row>
     <row r="133">
       <c r="A133" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>SKY ZONE WAYNE WILLOWBROOK NJ</t>
+          <t>SKY ZONE VISALIA</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>11184.3</v>
+        <v>16171.87</v>
       </c>
       <c r="D133" t="n">
-        <v>11184.3005</v>
+        <v>16171.8735</v>
       </c>
       <c r="E133" t="n">
-        <v>0.000499999998282874</v>
+        <v>0.003499999997075065</v>
       </c>
       <c r="F133" t="inlineStr">
         <is>
@@ -3623,21 +3623,21 @@
     </row>
     <row r="134">
       <c r="A134" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>SKY ZONE WHITBY</t>
+          <t>SKY ZONE WAYNE WILLOWBROOK NJ</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>5732.65</v>
+        <v>13912.71</v>
       </c>
       <c r="D134" t="n">
-        <v>5732.6539</v>
+        <v>13912.7083</v>
       </c>
       <c r="E134" t="n">
-        <v>0.003900000000612636</v>
+        <v>-0.001699999997072155</v>
       </c>
       <c r="F134" t="inlineStr">
         <is>
@@ -3647,21 +3647,21 @@
     </row>
     <row r="135">
       <c r="A135" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>SKY ZONE WILMINGTON NC</t>
+          <t>SKY ZONE WHITBY</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>7254.76</v>
+        <v>10611.83</v>
       </c>
       <c r="D135" t="n">
-        <v>7254.759100000001</v>
+        <v>10611.8286</v>
       </c>
       <c r="E135" t="n">
-        <v>-0.0008999999990919605</v>
+        <v>-0.001400000001012813</v>
       </c>
       <c r="F135" t="inlineStr">
         <is>
@@ -3671,21 +3671,21 @@
     </row>
     <row r="136">
       <c r="A136" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>SKY ZONE WOODBRIDGE</t>
+          <t>SKY ZONE WILMINGTON NC</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>4778.74</v>
+        <v>7904.3</v>
       </c>
       <c r="D136" t="n">
-        <v>4778.7433</v>
+        <v>7904.296800000001</v>
       </c>
       <c r="E136" t="n">
-        <v>0.003300000000308501</v>
+        <v>-0.003199999999196734</v>
       </c>
       <c r="F136" t="inlineStr">
         <is>
@@ -3695,21 +3695,21 @@
     </row>
     <row r="137">
       <c r="A137" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>SKY ZONE YONKERS</t>
+          <t>SKY ZONE WOODBRIDGE</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>19123.83</v>
+        <v>8149.95</v>
       </c>
       <c r="D137" t="n">
-        <v>19123.828</v>
+        <v>8149.9451</v>
       </c>
       <c r="E137" t="n">
-        <v>-0.002000000004045432</v>
+        <v>-0.004899999999906868</v>
       </c>
       <c r="F137" t="inlineStr">
         <is>
@@ -3719,23 +3719,47 @@
     </row>
     <row r="138">
       <c r="A138" s="1" t="n">
-        <v>46122</v>
+        <v>46145</v>
       </c>
       <c r="B138" t="inlineStr">
         <is>
+          <t>SKY ZONE YONKERS</t>
+        </is>
+      </c>
+      <c r="C138" t="n">
+        <v>16956.18</v>
+      </c>
+      <c r="D138" t="n">
+        <v>16956.1769</v>
+      </c>
+      <c r="E138" t="n">
+        <v>-0.003100000001722947</v>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>Match</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="1" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
           <t>SKY ZONE YONKERS CENTRAL PARK AVENUE NY</t>
         </is>
       </c>
-      <c r="C138" t="n">
-        <v>14462.7</v>
-      </c>
-      <c r="D138" t="n">
-        <v>14462.6979</v>
-      </c>
-      <c r="E138" t="n">
-        <v>-0.002099999999700231</v>
-      </c>
-      <c r="F138" t="inlineStr">
+      <c r="C139" t="n">
+        <v>19061.92</v>
+      </c>
+      <c r="D139" t="n">
+        <v>19061.9196</v>
+      </c>
+      <c r="E139" t="n">
+        <v>-0.0003999999971711077</v>
+      </c>
+      <c r="F139" t="inlineStr">
         <is>
           <t>Match</t>
         </is>
@@ -3774,7 +3798,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="3">
@@ -3784,7 +3808,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
final changes made to the project
</commit_message>
<xml_diff>
--- a/data/output/revenue_comparison.xlsx
+++ b/data/output/revenue_comparison.xlsx
@@ -455,7 +455,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -463,10 +463,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1157.49</v>
+        <v>2396.29</v>
       </c>
       <c r="D2" t="n">
-        <v>1157.49</v>
+        <v>2396.29</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -479,7 +479,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -487,13 +487,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>436.94</v>
+        <v>215.11</v>
       </c>
       <c r="D3" t="n">
-        <v>436.9422</v>
+        <v>215.1099</v>
       </c>
       <c r="E3" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -503,7 +503,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -511,13 +511,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>2030.74</v>
+        <v>1452.7</v>
       </c>
       <c r="D4" t="n">
-        <v>2030.7429</v>
+        <v>1452.6965</v>
       </c>
       <c r="E4" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -527,7 +527,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -535,13 +535,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>2753.33</v>
+        <v>3049.2</v>
       </c>
       <c r="D5" t="n">
-        <v>2753.329</v>
+        <v>3049.2045</v>
       </c>
       <c r="E5" t="n">
-        <v>0.001</v>
+        <v>0.005</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -551,7 +551,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -559,13 +559,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>2819.71</v>
+        <v>2518.27</v>
       </c>
       <c r="D6" t="n">
-        <v>2819.7105</v>
+        <v>2518.274</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>0.004</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -575,7 +575,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -583,10 +583,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>3918.97</v>
+        <v>2729.97</v>
       </c>
       <c r="D7" t="n">
-        <v>3918.9718</v>
+        <v>2729.9718</v>
       </c>
       <c r="E7" t="n">
         <v>0.002</v>
@@ -599,7 +599,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -607,10 +607,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>10079</v>
+        <v>6172</v>
       </c>
       <c r="D8" t="n">
-        <v>10079</v>
+        <v>6172</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
@@ -623,7 +623,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -631,10 +631,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1354.76</v>
+        <v>1327.06</v>
       </c>
       <c r="D9" t="n">
-        <v>1354.76</v>
+        <v>1327.06</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
@@ -647,7 +647,7 @@
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -655,13 +655,13 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>2023.59</v>
+        <v>1353.48</v>
       </c>
       <c r="D10" t="n">
-        <v>2025.3287</v>
+        <v>1351.7422</v>
       </c>
       <c r="E10" t="n">
-        <v>1.739</v>
+        <v>1.738</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -671,7 +671,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -679,13 +679,13 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>5504.2</v>
+        <v>6205.53</v>
       </c>
       <c r="D11" t="n">
-        <v>5504.196</v>
+        <v>6205.527099999998</v>
       </c>
       <c r="E11" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -695,7 +695,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -703,13 +703,13 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>4013.97</v>
+        <v>4004.09</v>
       </c>
       <c r="D12" t="n">
-        <v>4013.9659</v>
+        <v>4004.09</v>
       </c>
       <c r="E12" t="n">
-        <v>0.004</v>
+        <v>0</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -719,7 +719,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -727,13 +727,13 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>5669.1</v>
+        <v>4556.91</v>
       </c>
       <c r="D13" t="n">
-        <v>5669.1001</v>
+        <v>4556.9137</v>
       </c>
       <c r="E13" t="n">
-        <v>0</v>
+        <v>0.004</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -743,7 +743,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -751,13 +751,13 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>2157.32</v>
+        <v>2789.24</v>
       </c>
       <c r="D14" t="n">
-        <v>2157.3165</v>
+        <v>2789.239</v>
       </c>
       <c r="E14" t="n">
-        <v>0.004</v>
+        <v>0.001</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -767,7 +767,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -775,10 +775,10 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>898.41</v>
+        <v>2310.65</v>
       </c>
       <c r="D15" t="n">
-        <v>898.4129999999998</v>
+        <v>2310.6534</v>
       </c>
       <c r="E15" t="n">
         <v>0.003</v>
@@ -791,7 +791,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -799,13 +799,13 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1555.18</v>
+        <v>749.3</v>
       </c>
       <c r="D16" t="n">
-        <v>1555.1823</v>
+        <v>749.295</v>
       </c>
       <c r="E16" t="n">
-        <v>0.002</v>
+        <v>0.005</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -815,7 +815,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -823,10 +823,10 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>724.3200000000001</v>
+        <v>4041.01</v>
       </c>
       <c r="D17" t="n">
-        <v>724.3229000000001</v>
+        <v>4041.0073</v>
       </c>
       <c r="E17" t="n">
         <v>0.003</v>
@@ -839,7 +839,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>6673.42</v>
+        <v>7510.52</v>
       </c>
       <c r="D18" t="n">
-        <v>6673.42</v>
+        <v>7510.52</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
@@ -863,7 +863,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -871,10 +871,10 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2812.42</v>
+        <v>5540.82</v>
       </c>
       <c r="D19" t="n">
-        <v>2812.4183</v>
+        <v>5540.8223</v>
       </c>
       <c r="E19" t="n">
         <v>0.002</v>
@@ -887,7 +887,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -895,10 +895,10 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>1754.35</v>
+        <v>1900.26</v>
       </c>
       <c r="D20" t="n">
-        <v>1754.3477</v>
+        <v>1900.2577</v>
       </c>
       <c r="E20" t="n">
         <v>0.002</v>
@@ -911,7 +911,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -919,13 +919,13 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>3140.27</v>
+        <v>1949.83</v>
       </c>
       <c r="D21" t="n">
-        <v>3140.2672</v>
+        <v>1949.8301</v>
       </c>
       <c r="E21" t="n">
-        <v>0.003</v>
+        <v>0</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -935,7 +935,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -943,13 +943,13 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>2090.56</v>
+        <v>2571.29</v>
       </c>
       <c r="D22" t="n">
-        <v>2090.558</v>
+        <v>2571.2886</v>
       </c>
       <c r="E22" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -959,7 +959,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -967,13 +967,13 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>2907.21</v>
+        <v>3967.03</v>
       </c>
       <c r="D23" t="n">
-        <v>2907.2103</v>
+        <v>3967.0326</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>0.003</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -983,7 +983,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -991,13 +991,13 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>2639.31</v>
+        <v>1903.81</v>
       </c>
       <c r="D24" t="n">
-        <v>2639.31</v>
+        <v>1903.809</v>
       </c>
       <c r="E24" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -1007,7 +1007,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -1015,13 +1015,13 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>3196.29</v>
+        <v>3045.69</v>
       </c>
       <c r="D25" t="n">
-        <v>3196.2941</v>
+        <v>3045.6867</v>
       </c>
       <c r="E25" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -1031,7 +1031,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -1039,13 +1039,13 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>2650.66</v>
+        <v>1553.26</v>
       </c>
       <c r="D26" t="n">
-        <v>2650.664</v>
+        <v>1553.2566</v>
       </c>
       <c r="E26" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -1055,7 +1055,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -1063,13 +1063,13 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1522.25</v>
+        <v>2558.32</v>
       </c>
       <c r="D27" t="n">
-        <v>1522.2479</v>
+        <v>2558.3165</v>
       </c>
       <c r="E27" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -1079,7 +1079,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -1087,13 +1087,13 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>4080.51</v>
+        <v>2586.25</v>
       </c>
       <c r="D28" t="n">
-        <v>4080.5063</v>
+        <v>2586.2501</v>
       </c>
       <c r="E28" t="n">
-        <v>0.004</v>
+        <v>0</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -1103,7 +1103,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -1111,13 +1111,13 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>4521.09</v>
+        <v>3818.48</v>
       </c>
       <c r="D29" t="n">
-        <v>4521.0936</v>
+        <v>3818.4817</v>
       </c>
       <c r="E29" t="n">
-        <v>0.004</v>
+        <v>0.002</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -1127,7 +1127,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -1135,13 +1135,13 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>7810.24</v>
+        <v>9476.58</v>
       </c>
       <c r="D30" t="n">
-        <v>7810.240400000001</v>
+        <v>9476.579</v>
       </c>
       <c r="E30" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -1151,7 +1151,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -1159,13 +1159,13 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1540.34</v>
+        <v>3381.71</v>
       </c>
       <c r="D31" t="n">
-        <v>1540.3383</v>
+        <v>3381.7141</v>
       </c>
       <c r="E31" t="n">
-        <v>0.002</v>
+        <v>0.004</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -1175,7 +1175,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -1183,13 +1183,13 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>3011.89</v>
+        <v>2565.25</v>
       </c>
       <c r="D32" t="n">
-        <v>3011.8916</v>
+        <v>2565.2506</v>
       </c>
       <c r="E32" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -1199,7 +1199,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -1207,10 +1207,10 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>1907.75</v>
+        <v>1953.55</v>
       </c>
       <c r="D33" t="n">
-        <v>1907.7496</v>
+        <v>1953.55</v>
       </c>
       <c r="E33" t="n">
         <v>0</v>
@@ -1223,7 +1223,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -1231,13 +1231,13 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1273.32</v>
+        <v>1274.92</v>
       </c>
       <c r="D34" t="n">
-        <v>1273.3158</v>
+        <v>1274.9196</v>
       </c>
       <c r="E34" t="n">
-        <v>0.004</v>
+        <v>0</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -1247,7 +1247,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -1255,10 +1255,10 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>3763.34</v>
+        <v>1726.94</v>
       </c>
       <c r="D35" t="n">
-        <v>3763.3413</v>
+        <v>1726.9408</v>
       </c>
       <c r="E35" t="n">
         <v>0.001</v>
@@ -1271,7 +1271,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -1279,13 +1279,13 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>3991.56</v>
+        <v>2897.39</v>
       </c>
       <c r="D36" t="n">
-        <v>3991.5605</v>
+        <v>2897.3897</v>
       </c>
       <c r="E36" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -1295,7 +1295,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -1303,13 +1303,13 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>1469.76</v>
+        <v>3306.9</v>
       </c>
       <c r="D37" t="n">
-        <v>1469.7621</v>
+        <v>3306.8953</v>
       </c>
       <c r="E37" t="n">
-        <v>0.002</v>
+        <v>0.005</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
@@ -1319,7 +1319,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -1327,13 +1327,13 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>3207.58</v>
+        <v>3001.63</v>
       </c>
       <c r="D38" t="n">
-        <v>3207.5841</v>
+        <v>3001.6286</v>
       </c>
       <c r="E38" t="n">
-        <v>0.004</v>
+        <v>0.001</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
@@ -1343,7 +1343,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -1351,13 +1351,13 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>5122.81</v>
+        <v>5635.22</v>
       </c>
       <c r="D39" t="n">
-        <v>5122.811300000001</v>
+        <v>5635.217500000001</v>
       </c>
       <c r="E39" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
@@ -1367,7 +1367,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -1375,13 +1375,13 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>3896.31</v>
+        <v>3832.34</v>
       </c>
       <c r="D40" t="n">
-        <v>3896.309200000001</v>
+        <v>3832.3448</v>
       </c>
       <c r="E40" t="n">
-        <v>0.001</v>
+        <v>0.005</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
@@ -1391,7 +1391,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -1399,13 +1399,13 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>2581.77</v>
+        <v>4006.09</v>
       </c>
       <c r="D41" t="n">
-        <v>2581.77</v>
+        <v>4006.093</v>
       </c>
       <c r="E41" t="n">
-        <v>0</v>
+        <v>0.003</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
@@ -1415,7 +1415,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -1423,13 +1423,13 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>1082.49</v>
+        <v>1642.34</v>
       </c>
       <c r="D42" t="n">
-        <v>1082.487</v>
+        <v>1642.3377</v>
       </c>
       <c r="E42" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
@@ -1439,7 +1439,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -1447,13 +1447,13 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>1792.04</v>
+        <v>2927.35</v>
       </c>
       <c r="D43" t="n">
-        <v>1792.0421</v>
+        <v>2927.347200000001</v>
       </c>
       <c r="E43" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
@@ -1463,7 +1463,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -1471,13 +1471,13 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>2255.65</v>
+        <v>2564.5</v>
       </c>
       <c r="D44" t="n">
-        <v>2255.6544</v>
+        <v>2564.4952</v>
       </c>
       <c r="E44" t="n">
-        <v>0.004</v>
+        <v>0.005</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
@@ -1487,7 +1487,7 @@
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -1495,10 +1495,10 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>662.09</v>
+        <v>2025.17</v>
       </c>
       <c r="D45" t="n">
-        <v>662.09</v>
+        <v>2025.1702</v>
       </c>
       <c r="E45" t="n">
         <v>0</v>
@@ -1511,7 +1511,7 @@
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
@@ -1519,10 +1519,10 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>3110.23</v>
+        <v>3902.92</v>
       </c>
       <c r="D46" t="n">
-        <v>3110.23</v>
+        <v>3902.92</v>
       </c>
       <c r="E46" t="n">
         <v>0</v>
@@ -1535,7 +1535,7 @@
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -1543,13 +1543,13 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>2050.62</v>
+        <v>4230.06</v>
       </c>
       <c r="D47" t="n">
-        <v>2050.6242</v>
+        <v>4230.063</v>
       </c>
       <c r="E47" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
@@ -1559,7 +1559,7 @@
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
@@ -1567,10 +1567,10 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>3750.88</v>
+        <v>3007.73</v>
       </c>
       <c r="D48" t="n">
-        <v>3750.8808</v>
+        <v>3007.7313</v>
       </c>
       <c r="E48" t="n">
         <v>0.001</v>
@@ -1583,7 +1583,7 @@
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
@@ -1591,13 +1591,13 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>1821.77</v>
+        <v>2715.9</v>
       </c>
       <c r="D49" t="n">
-        <v>1821.7704</v>
+        <v>2715.8952</v>
       </c>
       <c r="E49" t="n">
-        <v>0</v>
+        <v>0.005</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
@@ -1607,7 +1607,7 @@
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
@@ -1615,13 +1615,13 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>2437.62</v>
+        <v>4095.88</v>
       </c>
       <c r="D50" t="n">
-        <v>2437.6194</v>
+        <v>4095.876</v>
       </c>
       <c r="E50" t="n">
-        <v>0.001</v>
+        <v>0.004</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
@@ -1631,7 +1631,7 @@
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
@@ -1639,13 +1639,13 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>1648.39</v>
+        <v>1763.11</v>
       </c>
       <c r="D51" t="n">
-        <v>1648.3913</v>
+        <v>1763.11</v>
       </c>
       <c r="E51" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
@@ -1655,7 +1655,7 @@
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
@@ -1663,13 +1663,13 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>1329.78</v>
+        <v>2031.96</v>
       </c>
       <c r="D52" t="n">
-        <v>1329.7759</v>
+        <v>2031.9604</v>
       </c>
       <c r="E52" t="n">
-        <v>0.004</v>
+        <v>0</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
@@ -1679,7 +1679,7 @@
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
@@ -1687,13 +1687,13 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>1505.68</v>
+        <v>2221.14</v>
       </c>
       <c r="D53" t="n">
-        <v>1505.6844</v>
+        <v>2221.1367</v>
       </c>
       <c r="E53" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
@@ -1703,7 +1703,7 @@
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
@@ -1711,13 +1711,13 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>4122.34</v>
+        <v>3137.61</v>
       </c>
       <c r="D54" t="n">
-        <v>4122.337699999999</v>
+        <v>3137.6108</v>
       </c>
       <c r="E54" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
@@ -1727,7 +1727,7 @@
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
@@ -1735,10 +1735,10 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>5253.28</v>
+        <v>4317.73</v>
       </c>
       <c r="D55" t="n">
-        <v>5253.2799</v>
+        <v>4317.73</v>
       </c>
       <c r="E55" t="n">
         <v>0</v>
@@ -1751,7 +1751,7 @@
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
@@ -1759,10 +1759,10 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>374.39</v>
+        <v>823.53</v>
       </c>
       <c r="D56" t="n">
-        <v>374.3933</v>
+        <v>823.5273</v>
       </c>
       <c r="E56" t="n">
         <v>0.003</v>
@@ -1775,7 +1775,7 @@
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
@@ -1783,13 +1783,13 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>7141.34</v>
+        <v>6471.5</v>
       </c>
       <c r="D57" t="n">
-        <v>7141.336</v>
+        <v>6471.500400000001</v>
       </c>
       <c r="E57" t="n">
-        <v>0.004</v>
+        <v>0</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
@@ -1799,7 +1799,7 @@
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
@@ -1807,13 +1807,13 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>8106.82</v>
+        <v>4837.58</v>
       </c>
       <c r="D58" t="n">
-        <v>8106.824600000001</v>
+        <v>4837.575500000001</v>
       </c>
       <c r="E58" t="n">
-        <v>0.005</v>
+        <v>0.004</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
@@ -1823,7 +1823,7 @@
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
@@ -1831,13 +1831,13 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>2373.24</v>
+        <v>3274.91</v>
       </c>
       <c r="D59" t="n">
-        <v>2373.2368</v>
+        <v>3274.9054</v>
       </c>
       <c r="E59" t="n">
-        <v>0.003</v>
+        <v>0.005</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
@@ -1847,7 +1847,7 @@
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
@@ -1855,13 +1855,13 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>1686.68</v>
+        <v>1500.2</v>
       </c>
       <c r="D60" t="n">
-        <v>1686.6805</v>
+        <v>1500.2036</v>
       </c>
       <c r="E60" t="n">
-        <v>0</v>
+        <v>0.004</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
@@ -1871,7 +1871,7 @@
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
@@ -1879,13 +1879,13 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>8260.700000000001</v>
+        <v>5060.5</v>
       </c>
       <c r="D61" t="n">
-        <v>8260.699000000001</v>
+        <v>5060.5025</v>
       </c>
       <c r="E61" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="F61" t="inlineStr">
         <is>
@@ -1895,7 +1895,7 @@
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
@@ -1903,13 +1903,13 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>4112.12</v>
+        <v>4006.39</v>
       </c>
       <c r="D62" t="n">
-        <v>4112.1205</v>
+        <v>4006.3899</v>
       </c>
       <c r="E62" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
@@ -1919,7 +1919,7 @@
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
@@ -1927,13 +1927,13 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>2629.88</v>
+        <v>2080.08</v>
       </c>
       <c r="D63" t="n">
-        <v>2629.88</v>
+        <v>2080.0818</v>
       </c>
       <c r="E63" t="n">
-        <v>0</v>
+        <v>0.002</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
@@ -1943,7 +1943,7 @@
     </row>
     <row r="64">
       <c r="A64" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
@@ -1951,13 +1951,13 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>1822.68</v>
+        <v>1547.86</v>
       </c>
       <c r="D64" t="n">
-        <v>1822.6838</v>
+        <v>1547.8611</v>
       </c>
       <c r="E64" t="n">
-        <v>0.004</v>
+        <v>0.001</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
@@ -1967,7 +1967,7 @@
     </row>
     <row r="65">
       <c r="A65" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
@@ -1975,13 +1975,13 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>1538.09</v>
+        <v>3500.61</v>
       </c>
       <c r="D65" t="n">
-        <v>1538.0911</v>
+        <v>3500.6064</v>
       </c>
       <c r="E65" t="n">
-        <v>0.001</v>
+        <v>0.004</v>
       </c>
       <c r="F65" t="inlineStr">
         <is>
@@ -1991,7 +1991,7 @@
     </row>
     <row r="66">
       <c r="A66" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
@@ -1999,13 +1999,13 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>1512.41</v>
+        <v>797.83</v>
       </c>
       <c r="D66" t="n">
-        <v>1512.4084</v>
+        <v>797.83</v>
       </c>
       <c r="E66" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="F66" t="inlineStr">
         <is>
@@ -2015,7 +2015,7 @@
     </row>
     <row r="67">
       <c r="A67" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
@@ -2023,13 +2023,13 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>1964.31</v>
+        <v>3603.12</v>
       </c>
       <c r="D67" t="n">
-        <v>1964.31</v>
+        <v>3603.1206</v>
       </c>
       <c r="E67" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="F67" t="inlineStr">
         <is>
@@ -2039,7 +2039,7 @@
     </row>
     <row r="68">
       <c r="A68" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
@@ -2047,13 +2047,13 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>2072.48</v>
+        <v>4049.4</v>
       </c>
       <c r="D68" t="n">
-        <v>2072.4821</v>
+        <v>4049.4033</v>
       </c>
       <c r="E68" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="F68" t="inlineStr">
         <is>
@@ -2063,7 +2063,7 @@
     </row>
     <row r="69">
       <c r="A69" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
@@ -2071,13 +2071,13 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>10961.36</v>
+        <v>8352.059999999999</v>
       </c>
       <c r="D69" t="n">
-        <v>10961.3649</v>
+        <v>8352.0607</v>
       </c>
       <c r="E69" t="n">
-        <v>0.005</v>
+        <v>0.001</v>
       </c>
       <c r="F69" t="inlineStr">
         <is>
@@ -2087,7 +2087,7 @@
     </row>
     <row r="70">
       <c r="A70" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
@@ -2095,13 +2095,13 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>3919.92</v>
+        <v>2915.89</v>
       </c>
       <c r="D70" t="n">
-        <v>3919.9203</v>
+        <v>2915.8932</v>
       </c>
       <c r="E70" t="n">
-        <v>0</v>
+        <v>0.003</v>
       </c>
       <c r="F70" t="inlineStr">
         <is>
@@ -2111,7 +2111,7 @@
     </row>
     <row r="71">
       <c r="A71" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
@@ -2119,13 +2119,13 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>4512.35</v>
+        <v>5490.71</v>
       </c>
       <c r="D71" t="n">
-        <v>4512.3529</v>
+        <v>5490.7104</v>
       </c>
       <c r="E71" t="n">
-        <v>0.003</v>
+        <v>0</v>
       </c>
       <c r="F71" t="inlineStr">
         <is>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="72">
       <c r="A72" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
@@ -2143,13 +2143,13 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>1035.76</v>
+        <v>1797.53</v>
       </c>
       <c r="D72" t="n">
-        <v>1035.7649</v>
+        <v>1797.53</v>
       </c>
       <c r="E72" t="n">
-        <v>0.005</v>
+        <v>0</v>
       </c>
       <c r="F72" t="inlineStr">
         <is>
@@ -2159,7 +2159,7 @@
     </row>
     <row r="73">
       <c r="A73" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
@@ -2167,13 +2167,13 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>2928.07</v>
+        <v>3944.69</v>
       </c>
       <c r="D73" t="n">
-        <v>2928.0661</v>
+        <v>3944.6881</v>
       </c>
       <c r="E73" t="n">
-        <v>0.004</v>
+        <v>0.002</v>
       </c>
       <c r="F73" t="inlineStr">
         <is>
@@ -2183,7 +2183,7 @@
     </row>
     <row r="74">
       <c r="A74" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
@@ -2191,13 +2191,13 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>3724.35</v>
+        <v>5837.44</v>
       </c>
       <c r="D74" t="n">
-        <v>3724.0307</v>
+        <v>6221.037399999999</v>
       </c>
       <c r="E74" t="n">
-        <v>0.319</v>
+        <v>383.597</v>
       </c>
       <c r="F74" t="inlineStr">
         <is>
@@ -2207,7 +2207,7 @@
     </row>
     <row r="75">
       <c r="A75" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
@@ -2215,13 +2215,13 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>864.5</v>
+        <v>1308.64</v>
       </c>
       <c r="D75" t="n">
-        <v>864.498</v>
+        <v>1308.6354</v>
       </c>
       <c r="E75" t="n">
-        <v>0.002</v>
+        <v>0.005</v>
       </c>
       <c r="F75" t="inlineStr">
         <is>
@@ -2231,7 +2231,7 @@
     </row>
     <row r="76">
       <c r="A76" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
@@ -2239,10 +2239,10 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>1664.56</v>
+        <v>896.28</v>
       </c>
       <c r="D76" t="n">
-        <v>1664.5624</v>
+        <v>896.2818</v>
       </c>
       <c r="E76" t="n">
         <v>0.002</v>
@@ -2255,7 +2255,7 @@
     </row>
     <row r="77">
       <c r="A77" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
@@ -2263,13 +2263,13 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>3155.55</v>
+        <v>2208.54</v>
       </c>
       <c r="D77" t="n">
-        <v>3155.552</v>
+        <v>2208.5374</v>
       </c>
       <c r="E77" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="F77" t="inlineStr">
         <is>
@@ -2279,7 +2279,7 @@
     </row>
     <row r="78">
       <c r="A78" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
@@ -2287,10 +2287,10 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>9884.290000000001</v>
+        <v>8288.889999999999</v>
       </c>
       <c r="D78" t="n">
-        <v>9884.292599999999</v>
+        <v>8288.8871</v>
       </c>
       <c r="E78" t="n">
         <v>0.003</v>
@@ -2303,7 +2303,7 @@
     </row>
     <row r="79">
       <c r="A79" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
@@ -2311,13 +2311,13 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>4263.09</v>
+        <v>6741.08</v>
       </c>
       <c r="D79" t="n">
-        <v>4263.089400000001</v>
+        <v>6741.084000000001</v>
       </c>
       <c r="E79" t="n">
-        <v>0.001</v>
+        <v>0.004</v>
       </c>
       <c r="F79" t="inlineStr">
         <is>
@@ -2327,7 +2327,7 @@
     </row>
     <row r="80">
       <c r="A80" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
@@ -2335,13 +2335,13 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>3084.77</v>
+        <v>2853.56</v>
       </c>
       <c r="D80" t="n">
-        <v>3084.7663</v>
+        <v>2853.56</v>
       </c>
       <c r="E80" t="n">
-        <v>0.004</v>
+        <v>0</v>
       </c>
       <c r="F80" t="inlineStr">
         <is>
@@ -2351,7 +2351,7 @@
     </row>
     <row r="81">
       <c r="A81" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
@@ -2359,10 +2359,10 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>6263.22</v>
+        <v>7028.63</v>
       </c>
       <c r="D81" t="n">
-        <v>6263.2237</v>
+        <v>7028.633800000001</v>
       </c>
       <c r="E81" t="n">
         <v>0.004</v>
@@ -2375,7 +2375,7 @@
     </row>
     <row r="82">
       <c r="A82" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
@@ -2383,13 +2383,13 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>3038.34</v>
+        <v>5345.89</v>
       </c>
       <c r="D82" t="n">
-        <v>3038.3363</v>
+        <v>5345.889999999999</v>
       </c>
       <c r="E82" t="n">
-        <v>0.004</v>
+        <v>0</v>
       </c>
       <c r="F82" t="inlineStr">
         <is>
@@ -2399,7 +2399,7 @@
     </row>
     <row r="83">
       <c r="A83" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
@@ -2407,13 +2407,13 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>1988.74</v>
+        <v>2363.34</v>
       </c>
       <c r="D83" t="n">
-        <v>1988.7351</v>
+        <v>2363.3444</v>
       </c>
       <c r="E83" t="n">
-        <v>0.005</v>
+        <v>0.004</v>
       </c>
       <c r="F83" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     </row>
     <row r="84">
       <c r="A84" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
@@ -2431,13 +2431,13 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>1189.38</v>
+        <v>2238.15</v>
       </c>
       <c r="D84" t="n">
-        <v>1189.38</v>
+        <v>2238.1506</v>
       </c>
       <c r="E84" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="F84" t="inlineStr">
         <is>
@@ -2447,7 +2447,7 @@
     </row>
     <row r="85">
       <c r="A85" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
@@ -2455,10 +2455,10 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>3022.08</v>
+        <v>3821.52</v>
       </c>
       <c r="D85" t="n">
-        <v>3022.0814</v>
+        <v>3821.5188</v>
       </c>
       <c r="E85" t="n">
         <v>0.001</v>
@@ -2471,7 +2471,7 @@
     </row>
     <row r="86">
       <c r="A86" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
@@ -2479,13 +2479,13 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>4060.57</v>
+        <v>5531.79</v>
       </c>
       <c r="D86" t="n">
-        <v>4060.5748</v>
+        <v>5531.7884</v>
       </c>
       <c r="E86" t="n">
-        <v>0.005</v>
+        <v>0.002</v>
       </c>
       <c r="F86" t="inlineStr">
         <is>
@@ -2495,7 +2495,7 @@
     </row>
     <row r="87">
       <c r="A87" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
@@ -2503,13 +2503,13 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>2352.17</v>
+        <v>4455.9</v>
       </c>
       <c r="D87" t="n">
-        <v>2352.1676</v>
+        <v>4455.8966</v>
       </c>
       <c r="E87" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="F87" t="inlineStr">
         <is>
@@ -2519,7 +2519,7 @@
     </row>
     <row r="88">
       <c r="A88" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
@@ -2527,13 +2527,13 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>3211.54</v>
+        <v>2047.18</v>
       </c>
       <c r="D88" t="n">
-        <v>3211.5405</v>
+        <v>2047.1766</v>
       </c>
       <c r="E88" t="n">
-        <v>0.001</v>
+        <v>0.003</v>
       </c>
       <c r="F88" t="inlineStr">
         <is>
@@ -2543,7 +2543,7 @@
     </row>
     <row r="89">
       <c r="A89" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
@@ -2551,13 +2551,13 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>2363</v>
+        <v>2937.75</v>
       </c>
       <c r="D89" t="n">
-        <v>2362.9973</v>
+        <v>2937.754</v>
       </c>
       <c r="E89" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
       <c r="F89" t="inlineStr">
         <is>
@@ -2567,7 +2567,7 @@
     </row>
     <row r="90">
       <c r="A90" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
@@ -2575,13 +2575,13 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>4522.58</v>
+        <v>3660.22</v>
       </c>
       <c r="D90" t="n">
-        <v>4522.5802</v>
+        <v>3660.2181</v>
       </c>
       <c r="E90" t="n">
-        <v>0</v>
+        <v>0.002</v>
       </c>
       <c r="F90" t="inlineStr">
         <is>
@@ -2591,7 +2591,7 @@
     </row>
     <row r="91">
       <c r="A91" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B91" t="inlineStr">
         <is>
@@ -2599,13 +2599,13 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>1332.57</v>
+        <v>1815.01</v>
       </c>
       <c r="D91" t="n">
-        <v>1332.5665</v>
+        <v>1815.0107</v>
       </c>
       <c r="E91" t="n">
-        <v>0.004</v>
+        <v>0.001</v>
       </c>
       <c r="F91" t="inlineStr">
         <is>
@@ -2615,7 +2615,7 @@
     </row>
     <row r="92">
       <c r="A92" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
@@ -2623,13 +2623,13 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>2370.28</v>
+        <v>1349.13</v>
       </c>
       <c r="D92" t="n">
-        <v>2370.2791</v>
+        <v>1349.13</v>
       </c>
       <c r="E92" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="F92" t="inlineStr">
         <is>
@@ -2639,7 +2639,7 @@
     </row>
     <row r="93">
       <c r="A93" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
@@ -2647,10 +2647,10 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>3131.48</v>
+        <v>3574.84</v>
       </c>
       <c r="D93" t="n">
-        <v>3131.4817</v>
+        <v>3574.838</v>
       </c>
       <c r="E93" t="n">
         <v>0.002</v>
@@ -2663,7 +2663,7 @@
     </row>
     <row r="94">
       <c r="A94" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
@@ -2671,13 +2671,13 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>1422.08</v>
+        <v>3024.6</v>
       </c>
       <c r="D94" t="n">
-        <v>1422.0788</v>
+        <v>3024.604400000001</v>
       </c>
       <c r="E94" t="n">
-        <v>0.001</v>
+        <v>0.004</v>
       </c>
       <c r="F94" t="inlineStr">
         <is>
@@ -2687,7 +2687,7 @@
     </row>
     <row r="95">
       <c r="A95" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
@@ -2695,10 +2695,10 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>3760.05</v>
+        <v>4195.91</v>
       </c>
       <c r="D95" t="n">
-        <v>3760.0496</v>
+        <v>4195.9101</v>
       </c>
       <c r="E95" t="n">
         <v>0</v>
@@ -2711,7 +2711,7 @@
     </row>
     <row r="96">
       <c r="A96" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
@@ -2719,13 +2719,13 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>779.66</v>
+        <v>2247.16</v>
       </c>
       <c r="D96" t="n">
-        <v>779.6605999999999</v>
+        <v>2247.1599</v>
       </c>
       <c r="E96" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="F96" t="inlineStr">
         <is>
@@ -2735,7 +2735,7 @@
     </row>
     <row r="97">
       <c r="A97" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
@@ -2743,10 +2743,10 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>4748.85</v>
+        <v>4701.05</v>
       </c>
       <c r="D97" t="n">
-        <v>4748.8516</v>
+        <v>4701.0517</v>
       </c>
       <c r="E97" t="n">
         <v>0.002</v>
@@ -2759,7 +2759,7 @@
     </row>
     <row r="98">
       <c r="A98" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
@@ -2767,13 +2767,13 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>1788</v>
+        <v>1528.59</v>
       </c>
       <c r="D98" t="n">
-        <v>1787.995</v>
+        <v>1528.59</v>
       </c>
       <c r="E98" t="n">
-        <v>0.005</v>
+        <v>0</v>
       </c>
       <c r="F98" t="inlineStr">
         <is>
@@ -2783,7 +2783,7 @@
     </row>
     <row r="99">
       <c r="A99" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
@@ -2791,13 +2791,13 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>1748.31</v>
+        <v>2124.14</v>
       </c>
       <c r="D99" t="n">
-        <v>1748.3139</v>
+        <v>2124.1392</v>
       </c>
       <c r="E99" t="n">
-        <v>0.004</v>
+        <v>0.001</v>
       </c>
       <c r="F99" t="inlineStr">
         <is>
@@ -2807,7 +2807,7 @@
     </row>
     <row r="100">
       <c r="A100" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
@@ -2815,13 +2815,13 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>4086.57</v>
+        <v>3489.86</v>
       </c>
       <c r="D100" t="n">
-        <v>4086.574100000001</v>
+        <v>3489.8551</v>
       </c>
       <c r="E100" t="n">
-        <v>0.004</v>
+        <v>0.005</v>
       </c>
       <c r="F100" t="inlineStr">
         <is>
@@ -2831,7 +2831,7 @@
     </row>
     <row r="101">
       <c r="A101" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
@@ -2839,13 +2839,13 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>4886.11</v>
+        <v>4185.03</v>
       </c>
       <c r="D101" t="n">
-        <v>4886.1108</v>
+        <v>4185.0268</v>
       </c>
       <c r="E101" t="n">
-        <v>0.001</v>
+        <v>0.003</v>
       </c>
       <c r="F101" t="inlineStr">
         <is>
@@ -2855,7 +2855,7 @@
     </row>
     <row r="102">
       <c r="A102" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
@@ -2863,13 +2863,13 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>2769.19</v>
+        <v>2582.65</v>
       </c>
       <c r="D102" t="n">
-        <v>2769.1909</v>
+        <v>2582.6481</v>
       </c>
       <c r="E102" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="F102" t="inlineStr">
         <is>
@@ -2879,7 +2879,7 @@
     </row>
     <row r="103">
       <c r="A103" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
@@ -2887,13 +2887,13 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>3472.06</v>
+        <v>3802.18</v>
       </c>
       <c r="D103" t="n">
-        <v>3472.064</v>
+        <v>3802.1794</v>
       </c>
       <c r="E103" t="n">
-        <v>0.004</v>
+        <v>0.001</v>
       </c>
       <c r="F103" t="inlineStr">
         <is>
@@ -2903,7 +2903,7 @@
     </row>
     <row r="104">
       <c r="A104" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
@@ -2911,13 +2911,13 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>4985.03</v>
+        <v>6605.03</v>
       </c>
       <c r="D104" t="n">
-        <v>4985.033299999999</v>
+        <v>6605.0316</v>
       </c>
       <c r="E104" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="F104" t="inlineStr">
         <is>
@@ -2927,7 +2927,7 @@
     </row>
     <row r="105">
       <c r="A105" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
@@ -2935,13 +2935,13 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>2254.22</v>
+        <v>2123.19</v>
       </c>
       <c r="D105" t="n">
-        <v>2254.2212</v>
+        <v>2123.19</v>
       </c>
       <c r="E105" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="F105" t="inlineStr">
         <is>
@@ -2951,7 +2951,7 @@
     </row>
     <row r="106">
       <c r="A106" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B106" t="inlineStr">
         <is>
@@ -2959,13 +2959,13 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>4357.84</v>
+        <v>3196.81</v>
       </c>
       <c r="D106" t="n">
-        <v>4357.836300000001</v>
+        <v>3196.8115</v>
       </c>
       <c r="E106" t="n">
-        <v>0.004</v>
+        <v>0.001</v>
       </c>
       <c r="F106" t="inlineStr">
         <is>
@@ -2975,7 +2975,7 @@
     </row>
     <row r="107">
       <c r="A107" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
@@ -2983,13 +2983,13 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>4162.25</v>
+        <v>7319.38</v>
       </c>
       <c r="D107" t="n">
-        <v>4162.2531</v>
+        <v>7319.3848</v>
       </c>
       <c r="E107" t="n">
-        <v>0.003</v>
+        <v>0.005</v>
       </c>
       <c r="F107" t="inlineStr">
         <is>
@@ -2999,7 +2999,7 @@
     </row>
     <row r="108">
       <c r="A108" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
@@ -3007,13 +3007,13 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>3139.34</v>
+        <v>4958.09</v>
       </c>
       <c r="D108" t="n">
-        <v>3139.3384</v>
+        <v>4958.0853</v>
       </c>
       <c r="E108" t="n">
-        <v>0.002</v>
+        <v>0.005</v>
       </c>
       <c r="F108" t="inlineStr">
         <is>
@@ -3023,7 +3023,7 @@
     </row>
     <row r="109">
       <c r="A109" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B109" t="inlineStr">
         <is>
@@ -3031,10 +3031,10 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>7358.67</v>
+        <v>10599.15</v>
       </c>
       <c r="D109" t="n">
-        <v>7358.6709</v>
+        <v>10599.1505</v>
       </c>
       <c r="E109" t="n">
         <v>0.001</v>
@@ -3047,7 +3047,7 @@
     </row>
     <row r="110">
       <c r="A110" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B110" t="inlineStr">
         <is>
@@ -3055,13 +3055,13 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>1438.14</v>
+        <v>1647.75</v>
       </c>
       <c r="D110" t="n">
-        <v>1438.1403</v>
+        <v>1647.7529</v>
       </c>
       <c r="E110" t="n">
-        <v>0</v>
+        <v>0.003</v>
       </c>
       <c r="F110" t="inlineStr">
         <is>
@@ -3071,7 +3071,7 @@
     </row>
     <row r="111">
       <c r="A111" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B111" t="inlineStr">
         <is>
@@ -3079,13 +3079,13 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>3031.55</v>
+        <v>5833</v>
       </c>
       <c r="D111" t="n">
-        <v>3031.5542</v>
+        <v>5832.9992</v>
       </c>
       <c r="E111" t="n">
-        <v>0.004</v>
+        <v>0.001</v>
       </c>
       <c r="F111" t="inlineStr">
         <is>
@@ -3095,7 +3095,7 @@
     </row>
     <row r="112">
       <c r="A112" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B112" t="inlineStr">
         <is>
@@ -3103,13 +3103,13 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>2387.61</v>
+        <v>2619.96</v>
       </c>
       <c r="D112" t="n">
-        <v>2387.6132</v>
+        <v>2619.9649</v>
       </c>
       <c r="E112" t="n">
-        <v>0.003</v>
+        <v>0.005</v>
       </c>
       <c r="F112" t="inlineStr">
         <is>
@@ -3119,7 +3119,7 @@
     </row>
     <row r="113">
       <c r="A113" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B113" t="inlineStr">
         <is>
@@ -3127,13 +3127,13 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>2021.62</v>
+        <v>4035.56</v>
       </c>
       <c r="D113" t="n">
-        <v>2021.6169</v>
+        <v>4035.5578</v>
       </c>
       <c r="E113" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="F113" t="inlineStr">
         <is>
@@ -3143,7 +3143,7 @@
     </row>
     <row r="114">
       <c r="A114" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B114" t="inlineStr">
         <is>
@@ -3151,13 +3151,13 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>2637.99</v>
+        <v>3499.11</v>
       </c>
       <c r="D114" t="n">
-        <v>2637.9907</v>
+        <v>3499.1068</v>
       </c>
       <c r="E114" t="n">
-        <v>0.001</v>
+        <v>0.003</v>
       </c>
       <c r="F114" t="inlineStr">
         <is>
@@ -3167,7 +3167,7 @@
     </row>
     <row r="115">
       <c r="A115" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B115" t="inlineStr">
         <is>
@@ -3175,13 +3175,13 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>5613.5</v>
+        <v>6172.57</v>
       </c>
       <c r="D115" t="n">
-        <v>5613.5031</v>
+        <v>6172.572</v>
       </c>
       <c r="E115" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="F115" t="inlineStr">
         <is>
@@ -3191,7 +3191,7 @@
     </row>
     <row r="116">
       <c r="A116" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B116" t="inlineStr">
         <is>
@@ -3199,13 +3199,13 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>3896.74</v>
+        <v>3454.44</v>
       </c>
       <c r="D116" t="n">
-        <v>3896.7365</v>
+        <v>3454.4412</v>
       </c>
       <c r="E116" t="n">
-        <v>0.003</v>
+        <v>0.001</v>
       </c>
       <c r="F116" t="inlineStr">
         <is>
@@ -3215,7 +3215,7 @@
     </row>
     <row r="117">
       <c r="A117" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B117" t="inlineStr">
         <is>
@@ -3223,13 +3223,13 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>2178.08</v>
+        <v>2132.96</v>
       </c>
       <c r="D117" t="n">
-        <v>2178.0764</v>
+        <v>2132.9629</v>
       </c>
       <c r="E117" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
       <c r="F117" t="inlineStr">
         <is>
@@ -3239,7 +3239,7 @@
     </row>
     <row r="118">
       <c r="A118" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B118" t="inlineStr">
         <is>
@@ -3247,13 +3247,13 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>3520.32</v>
+        <v>2420.29</v>
       </c>
       <c r="D118" t="n">
-        <v>3520.3171</v>
+        <v>2420.2859</v>
       </c>
       <c r="E118" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
       <c r="F118" t="inlineStr">
         <is>
@@ -3263,7 +3263,7 @@
     </row>
     <row r="119">
       <c r="A119" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B119" t="inlineStr">
         <is>
@@ -3271,13 +3271,13 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>3237.96</v>
+        <v>4227.62</v>
       </c>
       <c r="D119" t="n">
-        <v>3237.9601</v>
+        <v>4227.6168</v>
       </c>
       <c r="E119" t="n">
-        <v>0</v>
+        <v>0.003</v>
       </c>
       <c r="F119" t="inlineStr">
         <is>
@@ -3287,7 +3287,7 @@
     </row>
     <row r="120">
       <c r="A120" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B120" t="inlineStr">
         <is>
@@ -3295,13 +3295,13 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>4763.45</v>
+        <v>2695.49</v>
       </c>
       <c r="D120" t="n">
-        <v>4763.4524</v>
+        <v>2695.4909</v>
       </c>
       <c r="E120" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="F120" t="inlineStr">
         <is>
@@ -3311,7 +3311,7 @@
     </row>
     <row r="121">
       <c r="A121" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B121" t="inlineStr">
         <is>
@@ -3319,13 +3319,13 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>8207.92</v>
+        <v>9602.889999999999</v>
       </c>
       <c r="D121" t="n">
-        <v>8207.9195</v>
+        <v>9602.885399999999</v>
       </c>
       <c r="E121" t="n">
-        <v>0.001</v>
+        <v>0.005</v>
       </c>
       <c r="F121" t="inlineStr">
         <is>
@@ -3335,7 +3335,7 @@
     </row>
     <row r="122">
       <c r="A122" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B122" t="inlineStr">
         <is>
@@ -3343,13 +3343,13 @@
         </is>
       </c>
       <c r="C122" t="n">
-        <v>2220.47</v>
+        <v>2730.83</v>
       </c>
       <c r="D122" t="n">
-        <v>2220.4701</v>
+        <v>2730.8258</v>
       </c>
       <c r="E122" t="n">
-        <v>0</v>
+        <v>0.004</v>
       </c>
       <c r="F122" t="inlineStr">
         <is>
@@ -3359,7 +3359,7 @@
     </row>
     <row r="123">
       <c r="A123" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B123" t="inlineStr">
         <is>
@@ -3367,13 +3367,13 @@
         </is>
       </c>
       <c r="C123" t="n">
-        <v>2960.97</v>
+        <v>3528.18</v>
       </c>
       <c r="D123" t="n">
-        <v>2960.9707</v>
+        <v>3528.1756</v>
       </c>
       <c r="E123" t="n">
-        <v>0.001</v>
+        <v>0.004</v>
       </c>
       <c r="F123" t="inlineStr">
         <is>
@@ -3383,7 +3383,7 @@
     </row>
     <row r="124">
       <c r="A124" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B124" t="inlineStr">
         <is>
@@ -3391,13 +3391,13 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>21524.53</v>
+        <v>23383.75</v>
       </c>
       <c r="D124" t="n">
-        <v>21524.5298</v>
+        <v>23383.7532</v>
       </c>
       <c r="E124" t="n">
-        <v>0</v>
+        <v>0.003</v>
       </c>
       <c r="F124" t="inlineStr">
         <is>
@@ -3407,7 +3407,7 @@
     </row>
     <row r="125">
       <c r="A125" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B125" t="inlineStr">
         <is>
@@ -3415,13 +3415,13 @@
         </is>
       </c>
       <c r="C125" t="n">
-        <v>3394.68</v>
+        <v>3372.24</v>
       </c>
       <c r="D125" t="n">
-        <v>3506.5693</v>
+        <v>3223.2868</v>
       </c>
       <c r="E125" t="n">
-        <v>111.889</v>
+        <v>148.953</v>
       </c>
       <c r="F125" t="inlineStr">
         <is>
@@ -3431,7 +3431,7 @@
     </row>
     <row r="126">
       <c r="A126" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B126" t="inlineStr">
         <is>
@@ -3439,13 +3439,13 @@
         </is>
       </c>
       <c r="C126" t="n">
-        <v>7564.44</v>
+        <v>11455.17</v>
       </c>
       <c r="D126" t="n">
-        <v>7564.438</v>
+        <v>11455.1726</v>
       </c>
       <c r="E126" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="F126" t="inlineStr">
         <is>
@@ -3455,7 +3455,7 @@
     </row>
     <row r="127">
       <c r="A127" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B127" t="inlineStr">
         <is>
@@ -3463,10 +3463,10 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>4918.04</v>
+        <v>4414.03</v>
       </c>
       <c r="D127" t="n">
-        <v>4918.0374</v>
+        <v>4414.0334</v>
       </c>
       <c r="E127" t="n">
         <v>0.003</v>
@@ -3479,7 +3479,7 @@
     </row>
     <row r="128">
       <c r="A128" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B128" t="inlineStr">
         <is>
@@ -3487,13 +3487,13 @@
         </is>
       </c>
       <c r="C128" t="n">
-        <v>2569.72</v>
+        <v>2901.94</v>
       </c>
       <c r="D128" t="n">
-        <v>2569.7211</v>
+        <v>2901.9427</v>
       </c>
       <c r="E128" t="n">
-        <v>0.001</v>
+        <v>0.003</v>
       </c>
       <c r="F128" t="inlineStr">
         <is>
@@ -3503,7 +3503,7 @@
     </row>
     <row r="129">
       <c r="A129" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B129" t="inlineStr">
         <is>
@@ -3511,13 +3511,13 @@
         </is>
       </c>
       <c r="C129" t="n">
-        <v>3405.03</v>
+        <v>3066.73</v>
       </c>
       <c r="D129" t="n">
-        <v>3405.0315</v>
+        <v>3066.7316</v>
       </c>
       <c r="E129" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="F129" t="inlineStr">
         <is>
@@ -3527,7 +3527,7 @@
     </row>
     <row r="130">
       <c r="A130" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B130" t="inlineStr">
         <is>
@@ -3535,13 +3535,13 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>1472.4</v>
+        <v>2265.27</v>
       </c>
       <c r="D130" t="n">
-        <v>1472.3959</v>
+        <v>2265.27</v>
       </c>
       <c r="E130" t="n">
-        <v>0.004</v>
+        <v>0</v>
       </c>
       <c r="F130" t="inlineStr">
         <is>
@@ -3551,7 +3551,7 @@
     </row>
     <row r="131">
       <c r="A131" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B131" t="inlineStr">
         <is>
@@ -3559,13 +3559,13 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>5243.62</v>
+        <v>7462.3</v>
       </c>
       <c r="D131" t="n">
-        <v>5243.6192</v>
+        <v>7462.296400000001</v>
       </c>
       <c r="E131" t="n">
-        <v>0.001</v>
+        <v>0.004</v>
       </c>
       <c r="F131" t="inlineStr">
         <is>
@@ -3575,7 +3575,7 @@
     </row>
     <row r="132">
       <c r="A132" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B132" t="inlineStr">
         <is>
@@ -3583,13 +3583,13 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>2728.62</v>
+        <v>2017.46</v>
       </c>
       <c r="D132" t="n">
-        <v>2728.6175</v>
+        <v>2017.4646</v>
       </c>
       <c r="E132" t="n">
-        <v>0.003</v>
+        <v>0.005</v>
       </c>
       <c r="F132" t="inlineStr">
         <is>
@@ -3599,7 +3599,7 @@
     </row>
     <row r="133">
       <c r="A133" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B133" t="inlineStr">
         <is>
@@ -3607,10 +3607,10 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>2262.77</v>
+        <v>3109.72</v>
       </c>
       <c r="D133" t="n">
-        <v>2262.7693</v>
+        <v>3109.7191</v>
       </c>
       <c r="E133" t="n">
         <v>0.001</v>
@@ -3623,7 +3623,7 @@
     </row>
     <row r="134">
       <c r="A134" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B134" t="inlineStr">
         <is>
@@ -3631,13 +3631,13 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>2197.65</v>
+        <v>2684.14</v>
       </c>
       <c r="D134" t="n">
-        <v>2197.6514</v>
+        <v>2684.1398</v>
       </c>
       <c r="E134" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="F134" t="inlineStr">
         <is>
@@ -3647,7 +3647,7 @@
     </row>
     <row r="135">
       <c r="A135" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B135" t="inlineStr">
         <is>
@@ -3655,13 +3655,13 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>2102.99</v>
+        <v>2026.63</v>
       </c>
       <c r="D135" t="n">
-        <v>2102.986</v>
+        <v>2026.63</v>
       </c>
       <c r="E135" t="n">
-        <v>0.004</v>
+        <v>0</v>
       </c>
       <c r="F135" t="inlineStr">
         <is>
@@ -3671,7 +3671,7 @@
     </row>
     <row r="136">
       <c r="A136" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B136" t="inlineStr">
         <is>
@@ -3679,13 +3679,13 @@
         </is>
       </c>
       <c r="C136" t="n">
-        <v>4675.44</v>
+        <v>3442.41</v>
       </c>
       <c r="D136" t="n">
-        <v>4675.4446</v>
+        <v>3442.4076</v>
       </c>
       <c r="E136" t="n">
-        <v>0.005</v>
+        <v>0.002</v>
       </c>
       <c r="F136" t="inlineStr">
         <is>
@@ -3695,7 +3695,7 @@
     </row>
     <row r="137">
       <c r="A137" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B137" t="inlineStr">
         <is>
@@ -3703,13 +3703,13 @@
         </is>
       </c>
       <c r="C137" t="n">
-        <v>4110.45</v>
+        <v>2873.58</v>
       </c>
       <c r="D137" t="n">
-        <v>4110.4479</v>
+        <v>2873.5804</v>
       </c>
       <c r="E137" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="F137" t="inlineStr">
         <is>

</xml_diff>